<commit_message>
Settings: the page refuses to save (and says why) when the server is older than the page, instead of silently dropping the newer settings; number boxes take digits only (no e, + or -; no point in whole-number boxes), typing and pasting; two test cases; DevOps check that the API is current
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REIMSYS-test-cases.xlsx
+++ b/docs/REIMSYS-test-cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="697">
   <si>
     <t>REIMSYS: use cases and test cases</t>
   </si>
@@ -1767,6 +1767,32 @@
     <t>TC-102</t>
   </si>
   <si>
+    <t>Access &gt; Settings (and any number box in the app).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click a number box (keeping period, VAT rate, mail port, an amount on the receipt form).
+2. Type 1e+-2.5, or paste 1e5.</t>
+  </si>
+  <si>
+    <t>Only digits are accepted ( and the decimal point where decimals make sense). The letters e/E and the signs + and - cannot be typed or pasted. Whole-number boxes ignore the point.</t>
+  </si>
+  <si>
+    <t>TC-103</t>
+  </si>
+  <si>
+    <t>The web app is newer than the API (for example the API was not restarted after an update).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Access &gt; Settings.
+2. Change a value.</t>
+  </si>
+  <si>
+    <t>A red message says the page is newer than the server and lists the settings the server does not know; Save settings stays off, so nothing is silently dropped. After the API is rebuilt and restarted the message is gone and saving works.</t>
+  </si>
+  <si>
+    <t>TC-104</t>
+  </si>
+  <si>
     <t>Audit log</t>
   </si>
   <si>
@@ -1779,7 +1805,7 @@
     <t>Entries show who, what, when and (where relevant) the old and new values. Filters work together.</t>
   </si>
   <si>
-    <t>TC-103</t>
+    <t>TC-105</t>
   </si>
   <si>
     <t>Audit log open.</t>
@@ -1791,7 +1817,7 @@
     <t>A CSV with the filtered entries downloads.</t>
   </si>
   <si>
-    <t>TC-104</t>
+    <t>TC-106</t>
   </si>
   <si>
     <t>Access to the database server.</t>
@@ -1803,7 +1829,7 @@
     <t>The database refuses. The app can only read and add entries.</t>
   </si>
   <si>
-    <t>TC-105</t>
+    <t>TC-107</t>
   </si>
   <si>
     <t>A Checker opens evidence.</t>
@@ -1816,7 +1842,7 @@
     <t>Each view, download and print is recorded with the person and time.</t>
   </si>
   <si>
-    <t>TC-106</t>
+    <t>TC-108</t>
   </si>
   <si>
     <t>1. Profile &gt; Details: change name, phone, branch; Save.</t>
@@ -1825,7 +1851,7 @@
     <t>A message confirms; the new name shows in the side menu; a one-letter name is refused. The email cannot be changed here.</t>
   </si>
   <si>
-    <t>TC-107</t>
+    <t>TC-109</t>
   </si>
   <si>
     <t>Profile open.</t>
@@ -1837,7 +1863,7 @@
     <t>The photo is cropped square and shrunk, then accepted; the side menu and top bar show it at once.</t>
   </si>
   <si>
-    <t>TC-108</t>
+    <t>TC-110</t>
   </si>
   <si>
     <t>A profile photo exists.</t>
@@ -1850,7 +1876,7 @@
     <t>The new picture shows everywhere straight away. After Remove photo the initials come back and the button says Add photo; it is in the audit log.</t>
   </si>
   <si>
-    <t>TC-109</t>
+    <t>TC-111</t>
   </si>
   <si>
     <t xml:space="preserve">1. Profile &gt; Security: look at Where you are signed in.
@@ -1860,7 +1886,7 @@
     <t>This device is marked "This device". The other device is signed out.</t>
   </si>
   <si>
-    <t>TC-110</t>
+    <t>TC-112</t>
   </si>
   <si>
     <t>Profile &gt; Notifications.</t>
@@ -1872,7 +1898,7 @@
     <t>A message confirms each change. The required notices stay on.</t>
   </si>
   <si>
-    <t>TC-111</t>
+    <t>TC-113</t>
   </si>
   <si>
     <t>Profile &gt; Appearance.</t>
@@ -1884,7 +1910,7 @@
     <t>The whole app changes at once and the choice is kept after signing in again.</t>
   </si>
   <si>
-    <t>TC-112</t>
+    <t>TC-114</t>
   </si>
   <si>
     <t>Profile &gt; Activity.</t>
@@ -1896,7 +1922,7 @@
     <t>It lists your own recent actions only.</t>
   </si>
   <si>
-    <t>TC-113</t>
+    <t>TC-115</t>
   </si>
   <si>
     <t>Signed in as each role.</t>
@@ -1908,7 +1934,7 @@
     <t>The basics and "Your account" always show. Med Ref, Checker, Approver, Accounting and Super Admin each see only their own guide; the link bar matches.</t>
   </si>
   <si>
-    <t>TC-114</t>
+    <t>TC-116</t>
   </si>
   <si>
     <t>Keeping records</t>
@@ -1925,7 +1951,7 @@
     <t>It lists by month the paid and disapproved receipts older than the period (not approved-but-unpaid ones), with their total and files. The CSV matches. Nothing is deleted or hidden.</t>
   </si>
   <si>
-    <t>TC-115</t>
+    <t>TC-117</t>
   </si>
   <si>
     <t>Keeping period set.</t>
@@ -1937,7 +1963,7 @@
     <t>It is refused. Only administrators can see it. Each preview and download is in the audit log.</t>
   </si>
   <si>
-    <t>TC-116</t>
+    <t>TC-118</t>
   </si>
   <si>
     <t>Phone</t>
@@ -1952,7 +1978,7 @@
     <t>Every screen fits the width with no sideways scrolling; buttons are easy to tap; the bottom menu stays in place.</t>
   </si>
   <si>
-    <t>TC-117</t>
+    <t>TC-119</t>
   </si>
   <si>
     <t>Display</t>
@@ -1967,7 +1993,7 @@
     <t>Text is easy to read everywhere; nothing is hidden (white on white or black on black).</t>
   </si>
   <si>
-    <t>TC-118</t>
+    <t>TC-120</t>
   </si>
   <si>
     <t>1. Scroll any screen.</t>
@@ -1976,7 +2002,7 @@
     <t>The browser window itself never scrolls: the top bar and side menu stay put.</t>
   </si>
   <si>
-    <t>TC-119</t>
+    <t>TC-121</t>
   </si>
   <si>
     <t>A receipt with evidence.</t>
@@ -1988,7 +2014,7 @@
     <t>Both are refused. Evidence is served only through the app to people allowed to see it.</t>
   </si>
   <si>
-    <t>TC-120</t>
+    <t>TC-122</t>
   </si>
   <si>
     <t>1. Check the address uses https and look at the cookie.</t>
@@ -1997,7 +2023,7 @@
     <t>Only one cookie is used; it is HttpOnly and Secure. No outside scripts or fonts load.</t>
   </si>
   <si>
-    <t>TC-121</t>
+    <t>TC-123</t>
   </si>
   <si>
     <t>A form with text boxes.</t>
@@ -2009,7 +2035,7 @@
     <t>It shows as plain text and does not run.</t>
   </si>
   <si>
-    <t>TC-122</t>
+    <t>TC-124</t>
   </si>
   <si>
     <t>A signed-in session.</t>
@@ -2021,7 +2047,7 @@
     <t>The change is refused (cross-site requests are rejected).</t>
   </si>
   <si>
-    <t>TC-123</t>
+    <t>TC-125</t>
   </si>
   <si>
     <t>1. Run node scripts/preflight.mjs.</t>
@@ -2030,7 +2056,7 @@
     <t>No BLOCKER is listed: production mode, https address, a mail account, a real Super Admin, no demo accounts, and a recent backup.</t>
   </si>
   <si>
-    <t>TC-124</t>
+    <t>TC-126</t>
   </si>
   <si>
     <t>1. Run the backup. Then restore it into a spare database with node scripts/restore.mjs ... --db reimsys_restore_test.</t>
@@ -2039,7 +2065,7 @@
     <t>The backup holds the database and the files. The restored copy has the same number of receipts.</t>
   </si>
   <si>
-    <t>TC-125</t>
+    <t>TC-127</t>
   </si>
   <si>
     <t>1. Run node scripts/healthcheck.mjs while the API is running, then stop the API and run it again.</t>
@@ -2048,7 +2074,7 @@
     <t>It prints nothing when healthy, and names the problem (API not answering, low disk, old backup, stuck emails) when not.</t>
   </si>
   <si>
-    <t>TC-126</t>
+    <t>TC-128</t>
   </si>
   <si>
     <t>The server cannot send email.</t>
@@ -3294,7 +3320,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M127"/>
+  <dimension ref="A1:M129"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -7496,28 +7522,28 @@
         <v>562</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>563</v>
+        <v>29</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D103" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F103" s="10" t="s">
-        <v>158</v>
+        <v>216</v>
+      </c>
+      <c r="F103" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G103" s="8" t="s">
+        <v>563</v>
+      </c>
+      <c r="H103" s="8" t="s">
         <v>564</v>
       </c>
-      <c r="H103" s="8" t="s">
+      <c r="I103" s="8" t="s">
         <v>565</v>
-      </c>
-      <c r="I103" s="8" t="s">
-        <v>566</v>
       </c>
       <c r="J103" s="11" t="s">
         <v>162</v>
@@ -7534,31 +7560,31 @@
     </row>
     <row r="104" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>563</v>
+        <v>29</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D104" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F104" s="13" t="s">
-        <v>175</v>
+        <v>165</v>
+      </c>
+      <c r="F104" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G104" s="8" t="s">
+        <v>567</v>
+      </c>
+      <c r="H104" s="8" t="s">
         <v>568</v>
       </c>
-      <c r="H104" s="8" t="s">
+      <c r="I104" s="8" t="s">
         <v>569</v>
-      </c>
-      <c r="I104" s="8" t="s">
-        <v>570</v>
       </c>
       <c r="J104" s="11" t="s">
         <v>162</v>
@@ -7575,10 +7601,10 @@
     </row>
     <row r="105" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
+        <v>570</v>
+      </c>
+      <c r="B105" s="8" t="s">
         <v>571</v>
-      </c>
-      <c r="B105" s="8" t="s">
-        <v>563</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>112</v>
@@ -7587,7 +7613,7 @@
         <v>101</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>158</v>
@@ -7619,19 +7645,19 @@
         <v>575</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="C106" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="E106" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F106" s="10" t="s">
-        <v>158</v>
+      <c r="F106" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G106" s="8" t="s">
         <v>576</v>
@@ -7660,28 +7686,28 @@
         <v>579</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>119</v>
+        <v>571</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F107" s="13" t="s">
-        <v>175</v>
+        <v>170</v>
+      </c>
+      <c r="F107" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G107" s="8" t="s">
-        <v>121</v>
+        <v>580</v>
       </c>
       <c r="H107" s="8" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="I107" s="8" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J107" s="11" t="s">
         <v>162</v>
@@ -7698,16 +7724,16 @@
     </row>
     <row r="108" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>119</v>
+        <v>571</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E108" s="8" t="s">
         <v>157</v>
@@ -7716,13 +7742,13 @@
         <v>158</v>
       </c>
       <c r="G108" s="8" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H108" s="8" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I108" s="8" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="J108" s="11" t="s">
         <v>162</v>
@@ -7739,7 +7765,7 @@
     </row>
     <row r="109" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>119</v>
@@ -7757,7 +7783,7 @@
         <v>175</v>
       </c>
       <c r="G109" s="8" t="s">
-        <v>587</v>
+        <v>121</v>
       </c>
       <c r="H109" s="8" t="s">
         <v>588</v>
@@ -7789,22 +7815,22 @@
         <v>118</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E110" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F110" s="13" t="s">
-        <v>175</v>
+      <c r="F110" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>220</v>
+        <v>591</v>
       </c>
       <c r="H110" s="8" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="I110" s="8" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>162</v>
@@ -7821,7 +7847,7 @@
     </row>
     <row r="111" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B111" s="8" t="s">
         <v>119</v>
@@ -7830,22 +7856,22 @@
         <v>118</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E111" s="8" t="s">
         <v>157</v>
       </c>
       <c r="F111" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="H111" s="8" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="I111" s="8" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="J111" s="11" t="s">
         <v>162</v>
@@ -7862,7 +7888,7 @@
     </row>
     <row r="112" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B112" s="8" t="s">
         <v>119</v>
@@ -7874,13 +7900,13 @@
         <v>156</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F112" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G112" s="8" t="s">
-        <v>598</v>
+        <v>220</v>
       </c>
       <c r="H112" s="8" t="s">
         <v>599</v>
@@ -7947,16 +7973,16 @@
         <v>605</v>
       </c>
       <c r="B114" s="8" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="D114" s="8" t="s">
         <v>156</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
       <c r="F114" s="13" t="s">
         <v>190</v>
@@ -7988,28 +8014,28 @@
         <v>609</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>610</v>
+        <v>119</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="D115" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E115" s="8" t="s">
         <v>157</v>
       </c>
       <c r="F115" s="13" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="G115" s="8" t="s">
+        <v>610</v>
+      </c>
+      <c r="H115" s="8" t="s">
         <v>611</v>
       </c>
-      <c r="H115" s="8" t="s">
+      <c r="I115" s="8" t="s">
         <v>612</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>613</v>
       </c>
       <c r="J115" s="11" t="s">
         <v>162</v>
@@ -8026,31 +8052,31 @@
     </row>
     <row r="116" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="8" t="s">
+        <v>613</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D116" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F116" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="G116" s="8" t="s">
         <v>614</v>
       </c>
-      <c r="B116" s="8" t="s">
-        <v>610</v>
-      </c>
-      <c r="C116" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D116" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E116" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="F116" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G116" s="8" t="s">
+      <c r="H116" s="8" t="s">
         <v>615</v>
       </c>
-      <c r="H116" s="8" t="s">
+      <c r="I116" s="8" t="s">
         <v>616</v>
-      </c>
-      <c r="I116" s="8" t="s">
-        <v>617</v>
       </c>
       <c r="J116" s="11" t="s">
         <v>162</v>
@@ -8067,31 +8093,31 @@
     </row>
     <row r="117" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="B117" s="8" t="s">
         <v>618</v>
       </c>
-      <c r="B117" s="8" t="s">
+      <c r="C117" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F117" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="G117" s="8" t="s">
         <v>619</v>
       </c>
-      <c r="C117" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D117" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E117" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F117" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="G117" s="8" t="s">
+      <c r="H117" s="8" t="s">
         <v>620</v>
       </c>
-      <c r="H117" s="8" t="s">
+      <c r="I117" s="8" t="s">
         <v>621</v>
-      </c>
-      <c r="I117" s="8" t="s">
-        <v>622</v>
       </c>
       <c r="J117" s="11" t="s">
         <v>162</v>
@@ -8108,31 +8134,31 @@
     </row>
     <row r="118" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>624</v>
+        <v>618</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D118" s="8" t="s">
-        <v>156</v>
+        <v>101</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>197</v>
+        <v>313</v>
       </c>
       <c r="F118" s="13" t="s">
         <v>175</v>
       </c>
       <c r="G118" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="H118" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I118" s="8" t="s">
         <v>625</v>
-      </c>
-      <c r="H118" s="8" t="s">
-        <v>626</v>
-      </c>
-      <c r="I118" s="8" t="s">
-        <v>627</v>
       </c>
       <c r="J118" s="11" t="s">
         <v>162</v>
@@ -8149,25 +8175,25 @@
     </row>
     <row r="119" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="D119" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E119" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F119" s="13" t="s">
-        <v>175</v>
+      <c r="F119" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G119" s="8" t="s">
-        <v>491</v>
+        <v>628</v>
       </c>
       <c r="H119" s="8" t="s">
         <v>629</v>
@@ -8193,28 +8219,28 @@
         <v>631</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>170</v>
+        <v>632</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="D120" s="8" t="s">
         <v>156</v>
       </c>
       <c r="E120" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F120" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F120" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G120" s="8" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="H120" s="8" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="I120" s="8" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="J120" s="11" t="s">
         <v>162</v>
@@ -8231,31 +8257,31 @@
     </row>
     <row r="121" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>170</v>
+        <v>632</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="D121" s="8" t="s">
         <v>156</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F121" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F121" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G121" s="8" t="s">
-        <v>121</v>
+        <v>491</v>
       </c>
       <c r="H121" s="8" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="I121" s="8" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="J121" s="11" t="s">
         <v>162</v>
@@ -8272,7 +8298,7 @@
     </row>
     <row r="122" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B122" s="8" t="s">
         <v>170</v>
@@ -8286,17 +8312,17 @@
       <c r="E122" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F122" s="13" t="s">
-        <v>175</v>
+      <c r="F122" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G122" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="H122" s="8" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="I122" s="8" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="J122" s="11" t="s">
         <v>162</v>
@@ -8313,7 +8339,7 @@
     </row>
     <row r="123" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B123" s="8" t="s">
         <v>170</v>
@@ -8327,11 +8353,11 @@
       <c r="E123" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F123" s="13" t="s">
-        <v>175</v>
+      <c r="F123" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>643</v>
+        <v>121</v>
       </c>
       <c r="H123" s="8" t="s">
         <v>644</v>
@@ -8357,28 +8383,28 @@
         <v>646</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>137</v>
+        <v>28</v>
       </c>
       <c r="D124" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E124" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F124" s="10" t="s">
-        <v>158</v>
+        <v>170</v>
+      </c>
+      <c r="F124" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>141</v>
+        <v>647</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="I124" s="8" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="J124" s="11" t="s">
         <v>162</v>
@@ -8395,31 +8421,31 @@
     </row>
     <row r="125" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>137</v>
+        <v>28</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F125" s="10" t="s">
-        <v>158</v>
+        <v>170</v>
+      </c>
+      <c r="F125" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G125" s="8" t="s">
-        <v>141</v>
+        <v>651</v>
       </c>
       <c r="H125" s="8" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="I125" s="8" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="J125" s="11" t="s">
         <v>162</v>
@@ -8436,7 +8462,7 @@
     </row>
     <row r="126" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="B126" s="8" t="s">
         <v>138</v>
@@ -8450,17 +8476,17 @@
       <c r="E126" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F126" s="13" t="s">
-        <v>175</v>
+      <c r="F126" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G126" s="8" t="s">
         <v>141</v>
       </c>
       <c r="H126" s="8" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="I126" s="8" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="J126" s="11" t="s">
         <v>162</v>
@@ -8477,7 +8503,7 @@
     </row>
     <row r="127" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B127" s="8" t="s">
         <v>138</v>
@@ -8495,13 +8521,13 @@
         <v>158</v>
       </c>
       <c r="G127" s="8" t="s">
-        <v>656</v>
+        <v>141</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="I127" s="8" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="J127" s="11" t="s">
         <v>162</v>
@@ -8516,9 +8542,91 @@
         <v>1</v>
       </c>
     </row>
+    <row r="128" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="8" t="s">
+        <v>660</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D128" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E128" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F128" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="G128" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="H128" s="8" t="s">
+        <v>661</v>
+      </c>
+      <c r="I128" s="8" t="s">
+        <v>662</v>
+      </c>
+      <c r="J128" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="K128" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="L128" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="M128" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="8" t="s">
+        <v>663</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D129" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E129" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F129" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G129" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="H129" s="8" t="s">
+        <v>665</v>
+      </c>
+      <c r="I129" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="J129" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="K129" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="L129" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="M129" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M127"/>
-  <conditionalFormatting sqref="J2:J127">
+  <autoFilter ref="A1:M129"/>
+  <conditionalFormatting sqref="J2:J129">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -8530,10 +8638,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="J10:J127">
+    <dataValidation type="list" sqref="J10:J129">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J127">
+    <dataValidation type="list" sqref="J2:J129">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8554,7 +8662,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>1</v>
@@ -8580,22 +8688,22 @@
         <v>21</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8603,23 +8711,23 @@
         <v>155</v>
       </c>
       <c r="B3" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A3)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A3)</f>
         <v>10</v>
       </c>
       <c r="C3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A3,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A3,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A3,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A3,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>10</v>
       </c>
       <c r="G3" s="16">
@@ -8632,23 +8740,23 @@
         <v>201</v>
       </c>
       <c r="B4" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A4)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A4)</f>
         <v>7</v>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A4,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A4,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A4,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A4,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G4" s="16">
@@ -8661,23 +8769,23 @@
         <v>228</v>
       </c>
       <c r="B5" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A5)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A5)</f>
         <v>1</v>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A5,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A5,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A5,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A5,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G5" s="16">
@@ -8690,23 +8798,23 @@
         <v>233</v>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A6)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A6)</f>
         <v>4</v>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A6,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A6,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A6,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A6,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G6" s="16">
@@ -8719,23 +8827,23 @@
         <v>249</v>
       </c>
       <c r="B7" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A7)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A7)</f>
         <v>7</v>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A7,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A7,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A7,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A7,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G7" s="16">
@@ -8748,23 +8856,23 @@
         <v>272</v>
       </c>
       <c r="B8" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A8)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A8,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A8,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A8,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A8,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G8" s="16">
@@ -8777,23 +8885,23 @@
         <v>288</v>
       </c>
       <c r="B9" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A9)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A9)</f>
         <v>4</v>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A9,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A9,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A9,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A9,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G9" s="16">
@@ -8806,23 +8914,23 @@
         <v>43</v>
       </c>
       <c r="B10" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A10)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A10)</f>
         <v>4</v>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A10,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A10,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A10,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A10,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G10" s="16">
@@ -8835,23 +8943,23 @@
         <v>326</v>
       </c>
       <c r="B11" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A11)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A11)</f>
         <v>2</v>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A11,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A11,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A11,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A11,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G11" s="16">
@@ -8864,23 +8972,23 @@
         <v>335</v>
       </c>
       <c r="B12" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A12)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A12)</f>
         <v>1</v>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A12,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A12,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A12,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A12,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G12" s="16">
@@ -8893,23 +9001,23 @@
         <v>340</v>
       </c>
       <c r="B13" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A13)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A13)</f>
         <v>5</v>
       </c>
       <c r="C13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A13,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A13,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A13,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A13,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>5</v>
       </c>
       <c r="G13" s="16">
@@ -8922,23 +9030,23 @@
         <v>360</v>
       </c>
       <c r="B14" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A14)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A14)</f>
         <v>8</v>
       </c>
       <c r="C14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A14,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A14,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A14,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A14,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G14" s="16">
@@ -8951,23 +9059,23 @@
         <v>393</v>
       </c>
       <c r="B15" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A15)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A15)</f>
         <v>9</v>
       </c>
       <c r="C15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A15,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A15,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A15,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A15,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>9</v>
       </c>
       <c r="G15" s="16">
@@ -8980,23 +9088,23 @@
         <v>84</v>
       </c>
       <c r="B16" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A16)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A16)</f>
         <v>8</v>
       </c>
       <c r="C16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A16,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A16,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A16,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A16,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G16" s="16">
@@ -9009,23 +9117,23 @@
         <v>92</v>
       </c>
       <c r="B17" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A17)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A17)</f>
         <v>6</v>
       </c>
       <c r="C17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A17,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A17,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A17,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A17,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>6</v>
       </c>
       <c r="G17" s="16">
@@ -9038,23 +9146,23 @@
         <v>482</v>
       </c>
       <c r="B18" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A18)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A18)</f>
         <v>3</v>
       </c>
       <c r="C18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A18,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A18,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A18,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A18,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G18" s="16">
@@ -9067,23 +9175,23 @@
         <v>126</v>
       </c>
       <c r="B19" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A19)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A19,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A19,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A19,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A19,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G19" s="16">
@@ -9096,23 +9204,23 @@
         <v>499</v>
       </c>
       <c r="B20" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A20)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A20)</f>
         <v>7</v>
       </c>
       <c r="C20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A20,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A20,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A20,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A20,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G20" s="16">
@@ -9125,24 +9233,24 @@
         <v>29</v>
       </c>
       <c r="B21" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A21)</f>
-        <v>10</v>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A21)</f>
+        <v>12</v>
       </c>
       <c r="C21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A21,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A21,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A21,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A21,'Test cases'!$J$2:$J$127,"Not run")</f>
-        <v>10</v>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <v>12</v>
       </c>
       <c r="G21" s="16">
         <f>IF(B21=0,0,C21/B21)</f>
@@ -9151,26 +9259,26 @@
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="B22" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A22)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A22)</f>
         <v>4</v>
       </c>
       <c r="C22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A22,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A22,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A22,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A22,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G22" s="16">
@@ -9183,23 +9291,23 @@
         <v>119</v>
       </c>
       <c r="B23" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A23)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A23)</f>
         <v>7</v>
       </c>
       <c r="C23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A23,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A23,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A23,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A23,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G23" s="16">
@@ -9212,23 +9320,23 @@
         <v>133</v>
       </c>
       <c r="B24" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A24)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A24)</f>
         <v>1</v>
       </c>
       <c r="C24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A24,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A24,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A24,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A24,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G24" s="16">
@@ -9238,26 +9346,26 @@
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="B25" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A25)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A25)</f>
         <v>2</v>
       </c>
       <c r="C25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A25,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A25,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A25,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A25,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G25" s="16">
@@ -9267,26 +9375,26 @@
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="B26" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A26)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A26,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A26,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A26,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A26,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="16">
@@ -9296,26 +9404,26 @@
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="B27" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A27)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A27)</f>
         <v>2</v>
       </c>
       <c r="C27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A27,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A27,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A27,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A27,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G27" s="16">
@@ -9328,23 +9436,23 @@
         <v>170</v>
       </c>
       <c r="B28" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A28)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A28)</f>
         <v>4</v>
       </c>
       <c r="C28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A28,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A28,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A28,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A28,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G28" s="16">
@@ -9357,23 +9465,23 @@
         <v>138</v>
       </c>
       <c r="B29" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$127,$A29)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$129,$A29)</f>
         <v>4</v>
       </c>
       <c r="C29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A29,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A29,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A29,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$127,$A29,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G29" s="16">
@@ -9383,11 +9491,11 @@
     </row>
     <row r="30" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B30" s="18">
         <f>SUM(B3:B29)</f>
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C30" s="18">
         <f>SUM(C3:C29)</f>
@@ -9403,7 +9511,7 @@
       </c>
       <c r="F30" s="18">
         <f>SUM(F3:F29)</f>
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G30" s="19">
         <f>IF(B30=0,0,C30/B30)</f>
@@ -9412,7 +9520,7 @@
     </row>
     <row r="32" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>1</v>
@@ -9438,22 +9546,22 @@
         <v>12</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -9461,24 +9569,24 @@
         <v>158</v>
       </c>
       <c r="B34" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$127,A34)</f>
-        <v>63</v>
+        <f>COUNTIF('Test cases'!$F$2:$F$129,A34)</f>
+        <v>64</v>
       </c>
       <c r="C34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A34,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A34,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A34,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A34,'Test cases'!$J$2:$J$127,"Not run")</f>
-        <v>63</v>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <v>64</v>
       </c>
       <c r="G34" s="22">
         <f>IF(B34=0,0,C34/B34)</f>
@@ -9490,24 +9598,24 @@
         <v>175</v>
       </c>
       <c r="B35" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$127,A35)</f>
-        <v>45</v>
+        <f>COUNTIF('Test cases'!$F$2:$F$129,A35)</f>
+        <v>46</v>
       </c>
       <c r="C35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A35,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A35,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A35,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A35,'Test cases'!$J$2:$J$127,"Not run")</f>
-        <v>45</v>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <v>46</v>
       </c>
       <c r="G35" s="22">
         <f>IF(B35=0,0,C35/B35)</f>
@@ -9519,23 +9627,23 @@
         <v>190</v>
       </c>
       <c r="B36" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$127,A36)</f>
+        <f>COUNTIF('Test cases'!$F$2:$F$129,A36)</f>
         <v>18</v>
       </c>
       <c r="C36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A36,'Test cases'!$J$2:$J$127,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A36,'Test cases'!$J$2:$J$127,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A36,'Test cases'!$J$2:$J$127,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$127,$A36,'Test cases'!$J$2:$J$127,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Not run")</f>
         <v>18</v>
       </c>
       <c r="G36" s="22">
@@ -9545,7 +9653,7 @@
     </row>
     <row r="38" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
     </row>
   </sheetData>
@@ -9568,19 +9676,19 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9588,16 +9696,16 @@
         <v>44</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9605,16 +9713,16 @@
         <v>64</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9622,16 +9730,16 @@
         <v>77</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9639,16 +9747,16 @@
         <v>85</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9656,21 +9764,21 @@
         <v>101</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
How to read the invoice: a loading sign while a picture comes in, the old picture no longer left under the new tab's text, pictures of the same page fetched ahead, and a Try again when a picture cannot be loaded; test and workbook row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REIMSYS-test-cases.xlsx
+++ b/docs/REIMSYS-test-cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1945" uniqueCount="701">
   <si>
     <t>REIMSYS: use cases and test cases</t>
   </si>
@@ -855,6 +855,19 @@
     <t>TC-029</t>
   </si>
   <si>
+    <t>A phone on a slow connection (or throttled).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. On the invoice details step press How to read the invoice.
+2. Switch between the tabs (for example from The invoice to Withholding tax).</t>
+  </si>
+  <si>
+    <t>While a picture is coming in a spinner and "Loading the picture…" show and the old picture is not left under the new text. Tabs of the same page of the form appear at once (fetched ahead). If a picture cannot be loaded it says so and Try again works.</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
     <t>Evidence</t>
   </si>
   <si>
@@ -867,7 +880,7 @@
     <t>Each is accepted. The real file type is checked, not only its name.</t>
   </si>
   <si>
-    <t>TC-030</t>
+    <t>TC-031</t>
   </si>
   <si>
     <t xml:space="preserve">1. Rename a text or .exe file to .jpg and upload it.
@@ -877,7 +890,7 @@
     <t>Fake or oversized files and extra files are refused with a clear message.</t>
   </si>
   <si>
-    <t>TC-031</t>
+    <t>TC-032</t>
   </si>
   <si>
     <t>An earlier receipt with a photo exists.</t>
@@ -889,7 +902,7 @@
     <t>It is flagged as a possible duplicate (not silently accepted).</t>
   </si>
   <si>
-    <t>TC-032</t>
+    <t>TC-033</t>
   </si>
   <si>
     <t>Receipt with a photo.</t>
@@ -902,7 +915,7 @@
     <t>The whole picture shows first (also a very tall one). It zooms in to read details, can be moved around, returns with Fit, and Escape closes it.</t>
   </si>
   <si>
-    <t>TC-033</t>
+    <t>TC-034</t>
   </si>
   <si>
     <t>Scan</t>
@@ -919,7 +932,7 @@
     <t>The outline follows the receipt. The page is cut out straight. Use scan adds it to the receipt as a JPEG. Done lists the pages.</t>
   </si>
   <si>
-    <t>TC-034</t>
+    <t>TC-035</t>
   </si>
   <si>
     <t>A photo of a receipt.</t>
@@ -933,7 +946,7 @@
     <t>All four dots can be reached, even for a tall photo. The saved-page preview follows each change. Black &amp; white shows only black and white.</t>
   </si>
   <si>
-    <t>TC-035</t>
+    <t>TC-036</t>
   </si>
   <si>
     <t>A white receipt on a light desk.</t>
@@ -945,7 +958,7 @@
     <t>The receipt is outlined when it is clearly lighter than the desk; otherwise the corners start on the whole photo and can be dragged.</t>
   </si>
   <si>
-    <t>TC-036</t>
+    <t>TC-037</t>
   </si>
   <si>
     <t>The scan editor is open.</t>
@@ -957,7 +970,7 @@
     <t>All text is readable (nothing white on white), including when opened over the live camera screen.</t>
   </si>
   <si>
-    <t>TC-037</t>
+    <t>TC-038</t>
   </si>
   <si>
     <t>A phone.</t>
@@ -969,7 +982,7 @@
     <t>The date box is as wide as the other boxes and stays inside the card; the page does not scroll sideways.</t>
   </si>
   <si>
-    <t>TC-038</t>
+    <t>TC-039</t>
   </si>
   <si>
     <t>A Submitted receipt that nobody has opened yet.</t>
@@ -982,7 +995,7 @@
     <t>The receipt goes back to Draft and leaves the Checker's queue. It can be edited and submitted again.</t>
   </si>
   <si>
-    <t>TC-039</t>
+    <t>TC-040</t>
   </si>
   <si>
     <t>Permission</t>
@@ -997,7 +1010,7 @@
     <t>It is refused. A Med Ref can only see their own receipts.</t>
   </si>
   <si>
-    <t>TC-040</t>
+    <t>TC-041</t>
   </si>
   <si>
     <t>A receipt that is Checked or later.</t>
@@ -1009,7 +1022,7 @@
     <t>Editing is not offered (and the server refuses it). A paid receipt cannot be edited, withdrawn or deleted.</t>
   </si>
   <si>
-    <t>TC-041</t>
+    <t>TC-042</t>
   </si>
   <si>
     <t>The same receipt open in two windows.</t>
@@ -1022,7 +1035,7 @@
     <t>Window B is told the receipt changed and does not overwrite it (stale edits are refused).</t>
   </si>
   <si>
-    <t>TC-042</t>
+    <t>TC-043</t>
   </si>
   <si>
     <t>Import</t>
@@ -1039,7 +1052,7 @@
     <t>The preview lists each row and the error for the bad one. Only the valid rows are saved as Drafts. The bad row is not saved.</t>
   </si>
   <si>
-    <t>TC-043</t>
+    <t>TC-044</t>
   </si>
   <si>
     <t>On Import.</t>
@@ -1051,7 +1064,7 @@
     <t>It is refused with a clear message.</t>
   </si>
   <si>
-    <t>TC-044</t>
+    <t>TC-045</t>
   </si>
   <si>
     <t>Export</t>
@@ -1067,7 +1080,7 @@
     <t>The file contains the receipts the person may see, with invoice, VAT and withholding columns, and no category column.</t>
   </si>
   <si>
-    <t>TC-045</t>
+    <t>TC-046</t>
   </si>
   <si>
     <t>Receipt list</t>
@@ -1083,7 +1096,7 @@
     <t>The list and the counts on the status buttons follow every filter. Clear filters returns to everything.</t>
   </si>
   <si>
-    <t>TC-046</t>
+    <t>TC-047</t>
   </si>
   <si>
     <t>Several pages of receipts.</t>
@@ -1096,7 +1109,7 @@
     <t>The footer total is the amount of ALL matching receipts (every page), and changes with the filters. It equals the sum of the rows over all pages.</t>
   </si>
   <si>
-    <t>TC-047</t>
+    <t>TC-048</t>
   </si>
   <si>
     <t>Two Med Refs have receipts.</t>
@@ -1108,7 +1121,7 @@
     <t>Each sees only their own receipts and their own total.</t>
   </si>
   <si>
-    <t>TC-048</t>
+    <t>TC-049</t>
   </si>
   <si>
     <t xml:space="preserve">1. Open My receipts.
@@ -1118,7 +1131,7 @@
     <t>The search stays visible; the filters open and close behind a Filters button; status buttons scroll sideways in one row.</t>
   </si>
   <si>
-    <t>TC-049</t>
+    <t>TC-050</t>
   </si>
   <si>
     <t>A computer window at least 780 px tall.</t>
@@ -1130,7 +1143,7 @@
     <t>The page and menu stay still; only the rows scroll; column titles stay pinned; the footer stays at the bottom.</t>
   </si>
   <si>
-    <t>TC-050</t>
+    <t>TC-051</t>
   </si>
   <si>
     <t>Check</t>
@@ -1147,7 +1160,7 @@
     <t>Before the evidence is opened the buttons are locked with an explanation. Opening it is recorded. After opening, Mark checked works and the receipt becomes Checked; the Approver is told.</t>
   </si>
   <si>
-    <t>TC-051</t>
+    <t>TC-052</t>
   </si>
   <si>
     <t>A Submitted receipt.</t>
@@ -1162,7 +1175,7 @@
     <t>The receipt is Returned. The Med Ref gets a notice and an email that name the ticked problems and the note.</t>
   </si>
   <si>
-    <t>TC-052</t>
+    <t>TC-053</t>
   </si>
   <si>
     <t>The Return window is open.</t>
@@ -1175,7 +1188,7 @@
     <t>Both are refused: a problem or words are required.</t>
   </si>
   <si>
-    <t>TC-053</t>
+    <t>TC-054</t>
   </si>
   <si>
     <t>A Returned receipt with ticked problems.</t>
@@ -1189,7 +1202,7 @@
     <t>Fix opens the form on the right step. After submitting, the receipt is Submitted again and the ticked problems are cleared.</t>
   </si>
   <si>
-    <t>TC-054</t>
+    <t>TC-055</t>
   </si>
   <si>
     <t>The Checker has their own Submitted receipt (via another role).</t>
@@ -1201,7 +1214,7 @@
     <t>It is refused: reviewers cannot review their own receipts.</t>
   </si>
   <si>
-    <t>TC-055</t>
+    <t>TC-056</t>
   </si>
   <si>
     <t>A receipt open to the Checker.</t>
@@ -1214,7 +1227,7 @@
     <t>The comment appears on the receipt for both, with the author and time, and the other person gets a notice.</t>
   </si>
   <si>
-    <t>TC-056</t>
+    <t>TC-057</t>
   </si>
   <si>
     <t>Five Submitted receipts; evidence opened on three.</t>
@@ -1227,7 +1240,7 @@
     <t>The three are Checked. The other two are skipped and listed with the reason. At most 25 can be selected.</t>
   </si>
   <si>
-    <t>TC-057</t>
+    <t>TC-058</t>
   </si>
   <si>
     <t>A receipt that has waited several days.</t>
@@ -1239,7 +1252,7 @@
     <t>The waiting time shows (e.g. "6 days ago") and is highlighted when it passes the reminder limit.</t>
   </si>
   <si>
-    <t>TC-058</t>
+    <t>TC-059</t>
   </si>
   <si>
     <t>Decision</t>
@@ -1255,7 +1268,7 @@
     <t>The receipt is Approved, a reimbursement document (REIM-yyyy-nnnnnn) is created and can be downloaded and printed, and the Med Ref and Accounting are told.</t>
   </si>
   <si>
-    <t>TC-059</t>
+    <t>TC-060</t>
   </si>
   <si>
     <t>1. Press Disapprove and give a reason; confirm.</t>
@@ -1264,7 +1277,7 @@
     <t>The receipt is Disapproved with the reason shown to the Med Ref. Disapproved is final.</t>
   </si>
   <si>
-    <t>TC-060</t>
+    <t>TC-061</t>
   </si>
   <si>
     <t>The Disapprove or Reserve window is open.</t>
@@ -1276,7 +1289,7 @@
     <t>A reason (Disapprove) or a note (Reserve) is required.</t>
   </si>
   <si>
-    <t>TC-061</t>
+    <t>TC-062</t>
   </si>
   <si>
     <t xml:space="preserve">1. Press Reserve with a note.
@@ -1286,7 +1299,7 @@
     <t>It becomes Reserved (on hold) and the Med Ref is told; after Release it is back in the approval queue.</t>
   </si>
   <si>
-    <t>TC-062</t>
+    <t>TC-063</t>
   </si>
   <si>
     <t>1. Press Ask for more proof.</t>
@@ -1295,7 +1308,7 @@
     <t>The receipt goes back to the Med Ref, who can add proof and submit; it is then checked from the start.</t>
   </si>
   <si>
-    <t>TC-063</t>
+    <t>TC-064</t>
   </si>
   <si>
     <t>An Approved, unpaid receipt, within the undo time.</t>
@@ -1307,7 +1320,7 @@
     <t>It returns to Checked and the Med Ref is told to disregard the earlier approval. After the undo time (Access &gt; Settings) the button is gone.</t>
   </si>
   <si>
-    <t>TC-064</t>
+    <t>TC-065</t>
   </si>
   <si>
     <t>Several Checked receipts opened by the Approver.</t>
@@ -1319,7 +1332,7 @@
     <t>The ready ones are Approved with their documents. Any not ready are skipped with a reason.</t>
   </si>
   <si>
-    <t>TC-065</t>
+    <t>TC-066</t>
   </si>
   <si>
     <t>A Submitted (not yet Checked) receipt.</t>
@@ -1331,7 +1344,7 @@
     <t>The Approver cannot see or decide it: only checked receipts reach them.</t>
   </si>
   <si>
-    <t>TC-066</t>
+    <t>TC-067</t>
   </si>
   <si>
     <t>1. Try to approve a receipt by address or from the API.</t>
@@ -1340,7 +1353,7 @@
     <t>It is refused (no review rights).</t>
   </si>
   <si>
-    <t>TC-067</t>
+    <t>TC-068</t>
   </si>
   <si>
     <t>Approved receipts for two people.</t>
@@ -1352,7 +1365,7 @@
     <t>Receipts are grouped by person with the count and total; a header stays visible while scrolling; a footer shows people, receipts and total to pay.</t>
   </si>
   <si>
-    <t>TC-068</t>
+    <t>TC-069</t>
   </si>
   <si>
     <t>Approved receipts for one person.</t>
@@ -1367,7 +1380,7 @@
     <t>A payment number (PAY-yyyy-nnnnnn) is created. The receipts become Paid, show the payment card and cannot be edited. The Med Ref is emailed.</t>
   </si>
   <si>
-    <t>TC-069</t>
+    <t>TC-070</t>
   </si>
   <si>
     <t>The payment window is open.</t>
@@ -1379,7 +1392,7 @@
     <t>Each is refused with a clear message. A shortfall needs a reason. One payment covers one person only (up to 25 receipts).</t>
   </si>
   <si>
-    <t>TC-070</t>
+    <t>TC-071</t>
   </si>
   <si>
     <t>A Paid receipt.</t>
@@ -1391,7 +1404,7 @@
     <t>The receipt returns to Approved, the Med Ref is told, and the original payment record stays (it is never deleted).</t>
   </si>
   <si>
-    <t>TC-071</t>
+    <t>TC-072</t>
   </si>
   <si>
     <t>Paid receipts in a period.</t>
@@ -1403,7 +1416,7 @@
     <t>One row per paid receipt with the payment date, method and amounts.</t>
   </si>
   <si>
-    <t>TC-072</t>
+    <t>TC-073</t>
   </si>
   <si>
     <t>Signed in as Checker, Approver or Med Ref.</t>
@@ -1415,7 +1428,7 @@
     <t>The screen is not offered and the server refuses.</t>
   </si>
   <si>
-    <t>TC-073</t>
+    <t>TC-074</t>
   </si>
   <si>
     <t>Default rights.</t>
@@ -1427,7 +1440,7 @@
     <t>None of them are available to the Super Admin by default, so one person cannot run the whole chain.</t>
   </si>
   <si>
-    <t>TC-074</t>
+    <t>TC-075</t>
   </si>
   <si>
     <t>Access &gt; Settings.</t>
@@ -1439,7 +1452,7 @@
     <t>The methods are offered in the payment window. At most 12 methods; empty names refused.</t>
   </si>
   <si>
-    <t>TC-075</t>
+    <t>TC-076</t>
   </si>
   <si>
     <t>Approved receipts in the month.</t>
@@ -1454,7 +1467,7 @@
     <t>The count and total match the Approved (and Paid) receipts in the range. The report opens in the viewer with totals, by-type breakdown and the record table.</t>
   </si>
   <si>
-    <t>TC-076</t>
+    <t>TC-077</t>
   </si>
   <si>
     <t>A report exists.</t>
@@ -1466,7 +1479,7 @@
     <t>All three open and carry the same records and totals.</t>
   </si>
   <si>
-    <t>TC-077</t>
+    <t>TC-078</t>
   </si>
   <si>
     <t>On Reports.</t>
@@ -1478,7 +1491,7 @@
     <t>The first shows "Choose a valid date range"; the second disables Generate.</t>
   </si>
   <si>
-    <t>TC-078</t>
+    <t>TC-079</t>
   </si>
   <si>
     <t>Approved receipts for several people and types.</t>
@@ -1490,7 +1503,7 @@
     <t>Only matching records appear; pending, returned and disapproved receipts are never included.</t>
   </si>
   <si>
-    <t>TC-079</t>
+    <t>TC-080</t>
   </si>
   <si>
     <t>Two people made reports.</t>
@@ -1502,7 +1515,7 @@
     <t>A person sees only reports they made (an administrator may see more).</t>
   </si>
   <si>
-    <t>TC-080</t>
+    <t>TC-081</t>
   </si>
   <si>
     <t>A report with many rows.</t>
@@ -1514,7 +1527,7 @@
     <t>Column titles, the first column and the Total row stay in view; the page does not scroll.</t>
   </si>
   <si>
-    <t>TC-081</t>
+    <t>TC-082</t>
   </si>
   <si>
     <t>Dashboard</t>
@@ -1529,7 +1542,7 @@
     <t>Each role sees its own tiles and queue (Checker: To check; Approver: To decide; Accounting: To pay; Med Ref: Needs your action; Super Admin: Waiting for review). The highlighted first tile is the queue.</t>
   </si>
   <si>
-    <t>TC-082</t>
+    <t>TC-083</t>
   </si>
   <si>
     <t>Receipts in several statuses.</t>
@@ -1541,7 +1554,7 @@
     <t>The Receipts list opens already filtered to that status.</t>
   </si>
   <si>
-    <t>TC-083</t>
+    <t>TC-084</t>
   </si>
   <si>
     <t>A computer.</t>
@@ -1553,7 +1566,7 @@
     <t>It fits the window: the queue and Recent activity scroll inside their cards; the greeting is one line.</t>
   </si>
   <si>
-    <t>TC-084</t>
+    <t>TC-085</t>
   </si>
   <si>
     <t>A Med Ref with a receipt in review.</t>
@@ -1566,7 +1579,7 @@
     <t>The bell count increases; the notice names the receipt and opens it.</t>
   </si>
   <si>
-    <t>TC-085</t>
+    <t>TC-086</t>
   </si>
   <si>
     <t>Email</t>
@@ -1582,7 +1595,7 @@
     <t>One email arrives for each event with the right wording and a link button (https servers). Each shows status "sent" with the mail server's answer.</t>
   </si>
   <si>
-    <t>TC-086</t>
+    <t>TC-087</t>
   </si>
   <si>
     <t>Demo accounts on example.com.</t>
@@ -1594,7 +1607,7 @@
     <t>Nothing is sent. The Email log shows "logged" with "Example address, not a real mailbox".</t>
   </si>
   <si>
-    <t>TC-087</t>
+    <t>TC-088</t>
   </si>
   <si>
     <t>Access &gt; Email.</t>
@@ -1607,7 +1620,7 @@
     <t>Test connection reports success without sending. The test email arrives and shows "sent".</t>
   </si>
   <si>
-    <t>TC-088</t>
+    <t>TC-089</t>
   </si>
   <si>
     <t>1. Press Run full check.</t>
@@ -1616,7 +1629,7 @@
     <t>Five steps are listed (account, password key, server name, ports, login) each with a tick or a cross and, for a failure, what to do. Nothing is sent. Running it is in the audit log.</t>
   </si>
   <si>
-    <t>TC-089</t>
+    <t>TC-090</t>
   </si>
   <si>
     <t>A failed email in the log.</t>
@@ -1628,7 +1641,7 @@
     <t>It is queued again and its status updates.</t>
   </si>
   <si>
-    <t>TC-090</t>
+    <t>TC-091</t>
   </si>
   <si>
     <t>Receipts waiting several days.</t>
@@ -1640,7 +1653,7 @@
     <t>The Checker, Approver, Accounting and Med Ref get reminders only for what is waiting longer than the days set; a receipt that has not waited long gets none.</t>
   </si>
   <si>
-    <t>TC-091</t>
+    <t>TC-092</t>
   </si>
   <si>
     <t>Access &gt; Email templates.</t>
@@ -1652,7 +1665,7 @@
     <t>The change shows in the sample; unknown placeholders are refused.</t>
   </si>
   <si>
-    <t>TC-092</t>
+    <t>TC-093</t>
   </si>
   <si>
     <t xml:space="preserve">1. Access &gt; Users &gt; Add user (name, email, role).
@@ -1662,7 +1675,7 @@
     <t>The user appears in the list as Invited. They can sign in with the temporary password and must choose their own.</t>
   </si>
   <si>
-    <t>TC-093</t>
+    <t>TC-094</t>
   </si>
   <si>
     <t>A user with receipts.</t>
@@ -1675,7 +1688,7 @@
     <t>The user is signed out at once and cannot sign in; their receipts and history stay. They can be switched on again.</t>
   </si>
   <si>
-    <t>TC-094</t>
+    <t>TC-095</t>
   </si>
   <si>
     <t>A locked or forgotten account.</t>
@@ -1687,7 +1700,7 @@
     <t>A new temporary password is shown once and other sessions end; Unlock lets the person try again. Both are in the audit log.</t>
   </si>
   <si>
-    <t>TC-095</t>
+    <t>TC-096</t>
   </si>
   <si>
     <t>One active Super Admin only.</t>
@@ -1699,7 +1712,7 @@
     <t>It is refused: there must always be an active administrator.</t>
   </si>
   <si>
-    <t>TC-096</t>
+    <t>TC-097</t>
   </si>
   <si>
     <t>Roles and permissions tab.</t>
@@ -1712,7 +1725,7 @@
     <t>The change applies on their next action and is in the audit log. Locked rights (check, approve, pay, manage users/roles/settings) cannot be unticked.</t>
   </si>
   <si>
-    <t>TC-097</t>
+    <t>TC-098</t>
   </si>
   <si>
     <t>Roles tab.</t>
@@ -1724,7 +1737,7 @@
     <t>The role can be given to users and they see only what it allows (menu and Help guides follow the rights).</t>
   </si>
   <si>
-    <t>TC-098</t>
+    <t>TC-099</t>
   </si>
   <si>
     <t xml:space="preserve">1. Change a form rule (for example turn off "Accept receipts without a BIR invoice") and Save.
@@ -1734,7 +1747,7 @@
     <t>The "No" answer is no longer offered. Reset everything to default restores the starting values.</t>
   </si>
   <si>
-    <t>TC-099</t>
+    <t>TC-100</t>
   </si>
   <si>
     <t>1. Enter a value outside the allowed range (for example 0 for the undo time).</t>
@@ -1743,7 +1756,7 @@
     <t>The box shows an error; Save stays off.</t>
   </si>
   <si>
-    <t>TC-100</t>
+    <t>TC-101</t>
   </si>
   <si>
     <t>Access &gt; Company.</t>
@@ -1755,7 +1768,7 @@
     <t>They appear on documents, reports and emails.</t>
   </si>
   <si>
-    <t>TC-101</t>
+    <t>TC-102</t>
   </si>
   <si>
     <t>1. Open /access and /audit by address.</t>
@@ -1764,7 +1777,7 @@
     <t>Both send the person back to the Dashboard.</t>
   </si>
   <si>
-    <t>TC-102</t>
+    <t>TC-103</t>
   </si>
   <si>
     <t>Access &gt; Settings (and any number box in the app).</t>
@@ -1777,7 +1790,7 @@
     <t>Only digits are accepted ( and the decimal point where decimals make sense). The letters e/E and the signs + and - cannot be typed or pasted. Whole-number boxes ignore the point.</t>
   </si>
   <si>
-    <t>TC-103</t>
+    <t>TC-104</t>
   </si>
   <si>
     <t>The web app is newer than the API (for example the API was not restarted after an update).</t>
@@ -1790,7 +1803,7 @@
     <t>A red message says the page is newer than the server and lists the settings the server does not know. Those settings are hidden (no empty "Required" boxes), the other settings still change and save, and nothing is silently dropped. After the API is rebuilt and restarted the message is gone and every setting shows and saves.</t>
   </si>
   <si>
-    <t>TC-104</t>
+    <t>TC-105</t>
   </si>
   <si>
     <t>Audit log</t>
@@ -1805,7 +1818,7 @@
     <t>Entries show who, what, when and (where relevant) the old and new values. Filters work together.</t>
   </si>
   <si>
-    <t>TC-105</t>
+    <t>TC-106</t>
   </si>
   <si>
     <t>Audit log open.</t>
@@ -1817,7 +1830,7 @@
     <t>A CSV with the filtered entries downloads.</t>
   </si>
   <si>
-    <t>TC-106</t>
+    <t>TC-107</t>
   </si>
   <si>
     <t>Access to the database server.</t>
@@ -1829,7 +1842,7 @@
     <t>The database refuses. The app can only read and add entries.</t>
   </si>
   <si>
-    <t>TC-107</t>
+    <t>TC-108</t>
   </si>
   <si>
     <t>A Checker opens evidence.</t>
@@ -1842,7 +1855,7 @@
     <t>Each view, download and print is recorded with the person and time.</t>
   </si>
   <si>
-    <t>TC-108</t>
+    <t>TC-109</t>
   </si>
   <si>
     <t>1. Profile &gt; Details: change name, phone, branch; Save.</t>
@@ -1851,7 +1864,7 @@
     <t>A message confirms; the new name shows in the side menu; a one-letter name is refused. The email cannot be changed here.</t>
   </si>
   <si>
-    <t>TC-109</t>
+    <t>TC-110</t>
   </si>
   <si>
     <t>Profile open.</t>
@@ -1863,7 +1876,7 @@
     <t>The photo is cropped square and shrunk, then accepted; the side menu and top bar show it at once.</t>
   </si>
   <si>
-    <t>TC-110</t>
+    <t>TC-111</t>
   </si>
   <si>
     <t>A profile photo exists.</t>
@@ -1876,7 +1889,7 @@
     <t>The new picture shows everywhere straight away. After Remove photo the initials come back and the button says Add photo; it is in the audit log.</t>
   </si>
   <si>
-    <t>TC-111</t>
+    <t>TC-112</t>
   </si>
   <si>
     <t xml:space="preserve">1. Profile &gt; Security: look at Where you are signed in.
@@ -1886,7 +1899,7 @@
     <t>This device is marked "This device". The other device is signed out.</t>
   </si>
   <si>
-    <t>TC-112</t>
+    <t>TC-113</t>
   </si>
   <si>
     <t>Profile &gt; Notifications.</t>
@@ -1898,7 +1911,7 @@
     <t>A message confirms each change. The required notices stay on.</t>
   </si>
   <si>
-    <t>TC-113</t>
+    <t>TC-114</t>
   </si>
   <si>
     <t>Profile &gt; Appearance.</t>
@@ -1910,7 +1923,7 @@
     <t>The whole app changes at once and the choice is kept after signing in again.</t>
   </si>
   <si>
-    <t>TC-114</t>
+    <t>TC-115</t>
   </si>
   <si>
     <t>Profile &gt; Activity.</t>
@@ -1922,7 +1935,7 @@
     <t>It lists your own recent actions only.</t>
   </si>
   <si>
-    <t>TC-115</t>
+    <t>TC-116</t>
   </si>
   <si>
     <t>Signed in as each role.</t>
@@ -1934,7 +1947,7 @@
     <t>The basics and "Your account" always show. Med Ref, Checker, Approver, Accounting and Super Admin each see only their own guide; the link bar matches.</t>
   </si>
   <si>
-    <t>TC-116</t>
+    <t>TC-117</t>
   </si>
   <si>
     <t>Keeping records</t>
@@ -1951,7 +1964,7 @@
     <t>It lists by month the paid and disapproved receipts older than the period (not approved-but-unpaid ones), with their total and files. The CSV matches. Nothing is deleted or hidden.</t>
   </si>
   <si>
-    <t>TC-117</t>
+    <t>TC-118</t>
   </si>
   <si>
     <t>Keeping period set.</t>
@@ -1963,7 +1976,7 @@
     <t>It is refused. Only administrators can see it. Each preview and download is in the audit log.</t>
   </si>
   <si>
-    <t>TC-118</t>
+    <t>TC-119</t>
   </si>
   <si>
     <t>Phone</t>
@@ -1978,7 +1991,7 @@
     <t>Every screen fits the width with no sideways scrolling; buttons are easy to tap; the bottom menu stays in place.</t>
   </si>
   <si>
-    <t>TC-119</t>
+    <t>TC-120</t>
   </si>
   <si>
     <t>Display</t>
@@ -1993,7 +2006,7 @@
     <t>Text is easy to read everywhere; nothing is hidden (white on white or black on black).</t>
   </si>
   <si>
-    <t>TC-120</t>
+    <t>TC-121</t>
   </si>
   <si>
     <t>1. Scroll any screen.</t>
@@ -2002,7 +2015,7 @@
     <t>The browser window itself never scrolls: the top bar and side menu stay put.</t>
   </si>
   <si>
-    <t>TC-121</t>
+    <t>TC-122</t>
   </si>
   <si>
     <t>A receipt with evidence.</t>
@@ -2014,7 +2027,7 @@
     <t>Both are refused. Evidence is served only through the app to people allowed to see it.</t>
   </si>
   <si>
-    <t>TC-122</t>
+    <t>TC-123</t>
   </si>
   <si>
     <t>1. Check the address uses https and look at the cookie.</t>
@@ -2023,7 +2036,7 @@
     <t>Only one cookie is used; it is HttpOnly and Secure. No outside scripts or fonts load.</t>
   </si>
   <si>
-    <t>TC-123</t>
+    <t>TC-124</t>
   </si>
   <si>
     <t>A form with text boxes.</t>
@@ -2035,7 +2048,7 @@
     <t>It shows as plain text and does not run.</t>
   </si>
   <si>
-    <t>TC-124</t>
+    <t>TC-125</t>
   </si>
   <si>
     <t>A signed-in session.</t>
@@ -2047,7 +2060,7 @@
     <t>The change is refused (cross-site requests are rejected).</t>
   </si>
   <si>
-    <t>TC-125</t>
+    <t>TC-126</t>
   </si>
   <si>
     <t>1. Run node scripts/preflight.mjs.</t>
@@ -2056,7 +2069,7 @@
     <t>No BLOCKER is listed: production mode, https address, a mail account, a real Super Admin, no demo accounts, and a recent backup.</t>
   </si>
   <si>
-    <t>TC-126</t>
+    <t>TC-127</t>
   </si>
   <si>
     <t>1. Run the backup. Then restore it into a spare database with node scripts/restore.mjs ... --db reimsys_restore_test.</t>
@@ -2065,7 +2078,7 @@
     <t>The backup holds the database and the files. The restored copy has the same number of receipts.</t>
   </si>
   <si>
-    <t>TC-127</t>
+    <t>TC-128</t>
   </si>
   <si>
     <t>1. Run node scripts/healthcheck.mjs while the API is running, then stop the API and run it again.</t>
@@ -2074,7 +2087,7 @@
     <t>It prints nothing when healthy, and names the problem (API not answering, low disk, old backup, stuck emails) when not.</t>
   </si>
   <si>
-    <t>TC-128</t>
+    <t>TC-129</t>
   </si>
   <si>
     <t>The server cannot send email.</t>
@@ -3320,7 +3333,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4529,7 +4542,7 @@
         <v>271</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>272</v>
+        <v>249</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>42</v>
@@ -4538,19 +4551,19 @@
         <v>44</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G30" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="H30" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="I30" s="8" t="s">
         <v>274</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>275</v>
       </c>
       <c r="J30" s="11" t="s">
         <v>162</v>
@@ -4567,10 +4580,10 @@
     </row>
     <row r="31" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>276</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>272</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>42</v>
@@ -4579,19 +4592,19 @@
         <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J31" s="11" t="s">
         <v>162</v>
@@ -4608,10 +4621,10 @@
     </row>
     <row r="32" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>42</v>
@@ -4620,13 +4633,13 @@
         <v>44</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>175</v>
+        <v>216</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H32" s="8" t="s">
         <v>281</v>
@@ -4652,7 +4665,7 @@
         <v>283</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>42</v>
@@ -4663,8 +4676,8 @@
       <c r="E33" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>158</v>
+      <c r="F33" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>284</v>
@@ -4693,7 +4706,7 @@
         <v>287</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>42</v>
@@ -4708,13 +4721,13 @@
         <v>158</v>
       </c>
       <c r="G34" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="H34" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="H34" s="8" t="s">
+      <c r="I34" s="8" t="s">
         <v>290</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>291</v>
       </c>
       <c r="J34" s="11" t="s">
         <v>162</v>
@@ -4731,10 +4744,10 @@
     </row>
     <row r="35" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>288</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>42</v>
@@ -4775,7 +4788,7 @@
         <v>296</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>42</v>
@@ -4786,8 +4799,8 @@
       <c r="E36" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F36" s="13" t="s">
-        <v>175</v>
+      <c r="F36" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>297</v>
@@ -4816,7 +4829,7 @@
         <v>300</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>42</v>
@@ -4857,7 +4870,7 @@
         <v>304</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>249</v>
+        <v>292</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>42</v>
@@ -4866,7 +4879,7 @@
         <v>44</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F38" s="13" t="s">
         <v>175</v>
@@ -4898,7 +4911,7 @@
         <v>308</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>43</v>
+        <v>249</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>42</v>
@@ -4907,10 +4920,10 @@
         <v>44</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>309</v>
@@ -4948,19 +4961,19 @@
         <v>44</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>313</v>
+        <v>157</v>
       </c>
       <c r="F40" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G40" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="H40" s="8" t="s">
         <v>314</v>
       </c>
-      <c r="H40" s="8" t="s">
+      <c r="I40" s="8" t="s">
         <v>315</v>
-      </c>
-      <c r="I40" s="8" t="s">
-        <v>316</v>
       </c>
       <c r="J40" s="11" t="s">
         <v>162</v>
@@ -4977,7 +4990,7 @@
     </row>
     <row r="41" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B41" s="8" t="s">
         <v>43</v>
@@ -4989,7 +5002,7 @@
         <v>44</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>165</v>
+        <v>317</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>158</v>
@@ -5030,10 +5043,10 @@
         <v>44</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>175</v>
+        <v>165</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>322</v>
@@ -5062,10 +5075,10 @@
         <v>325</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>326</v>
+        <v>43</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>44</v>
@@ -5077,13 +5090,13 @@
         <v>175</v>
       </c>
       <c r="G43" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="H43" s="8" t="s">
         <v>327</v>
       </c>
-      <c r="H43" s="8" t="s">
+      <c r="I43" s="8" t="s">
         <v>328</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>329</v>
       </c>
       <c r="J43" s="11" t="s">
         <v>162</v>
@@ -5100,10 +5113,10 @@
     </row>
     <row r="44" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="B44" s="8" t="s">
         <v>330</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>326</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>56</v>
@@ -5112,10 +5125,10 @@
         <v>44</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>331</v>
@@ -5144,28 +5157,28 @@
         <v>334</v>
       </c>
       <c r="B45" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="G45" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="C45" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F45" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G45" s="8" t="s">
+      <c r="H45" s="8" t="s">
         <v>336</v>
       </c>
-      <c r="H45" s="8" t="s">
+      <c r="I45" s="8" t="s">
         <v>337</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>338</v>
       </c>
       <c r="J45" s="11" t="s">
         <v>162</v>
@@ -5182,13 +5195,13 @@
     </row>
     <row r="46" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B46" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="B46" s="8" t="s">
-        <v>340</v>
-      </c>
       <c r="C46" s="8" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>64</v>
@@ -5196,17 +5209,17 @@
       <c r="E46" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>158</v>
+      <c r="F46" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G46" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>341</v>
       </c>
-      <c r="H46" s="8" t="s">
+      <c r="I46" s="8" t="s">
         <v>342</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>343</v>
       </c>
       <c r="J46" s="11" t="s">
         <v>162</v>
@@ -5223,10 +5236,10 @@
     </row>
     <row r="47" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="B47" s="8" t="s">
         <v>344</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>340</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>62</v>
@@ -5267,16 +5280,16 @@
         <v>348</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>62</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>313</v>
+        <v>157</v>
       </c>
       <c r="F48" s="10" t="s">
         <v>158</v>
@@ -5308,7 +5321,7 @@
         <v>352</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>62</v>
@@ -5317,19 +5330,19 @@
         <v>44</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F49" s="13" t="s">
-        <v>175</v>
+        <v>317</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>305</v>
+        <v>353</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J49" s="11" t="s">
         <v>162</v>
@@ -5346,25 +5359,25 @@
     </row>
     <row r="50" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>62</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>197</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>356</v>
+        <v>309</v>
       </c>
       <c r="H50" s="8" t="s">
         <v>357</v>
@@ -5390,7 +5403,7 @@
         <v>359</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>360</v>
+        <v>344</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>62</v>
@@ -5399,19 +5412,19 @@
         <v>64</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G51" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="H51" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="H51" s="8" t="s">
+      <c r="I51" s="8" t="s">
         <v>362</v>
-      </c>
-      <c r="I51" s="8" t="s">
-        <v>363</v>
       </c>
       <c r="J51" s="11" t="s">
         <v>162</v>
@@ -5428,10 +5441,10 @@
     </row>
     <row r="52" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="B52" s="8" t="s">
         <v>364</v>
-      </c>
-      <c r="B52" s="8" t="s">
-        <v>360</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>62</v>
@@ -5472,7 +5485,7 @@
         <v>368</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>62</v>
@@ -5481,10 +5494,10 @@
         <v>64</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="F53" s="13" t="s">
-        <v>175</v>
+        <v>157</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>369</v>
@@ -5513,19 +5526,19 @@
         <v>372</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F54" s="10" t="s">
-        <v>158</v>
+        <v>216</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>373</v>
@@ -5554,16 +5567,16 @@
         <v>376</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>313</v>
+        <v>157</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>158</v>
@@ -5595,7 +5608,7 @@
         <v>380</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>62</v>
@@ -5604,10 +5617,10 @@
         <v>64</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F56" s="13" t="s">
-        <v>175</v>
+        <v>317</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>381</v>
@@ -5636,10 +5649,10 @@
         <v>384</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>64</v>
@@ -5677,10 +5690,10 @@
         <v>388</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>64</v>
@@ -5718,28 +5731,28 @@
         <v>392</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>393</v>
+        <v>364</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F59" s="10" t="s">
-        <v>158</v>
+      <c r="F59" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G59" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="H59" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="H59" s="8" t="s">
+      <c r="I59" s="8" t="s">
         <v>395</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>396</v>
       </c>
       <c r="J59" s="11" t="s">
         <v>162</v>
@@ -5756,10 +5769,10 @@
     </row>
     <row r="60" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="B60" s="8" t="s">
         <v>397</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>393</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>76</v>
@@ -5774,13 +5787,13 @@
         <v>158</v>
       </c>
       <c r="G60" s="8" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="H60" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I60" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>162</v>
@@ -5797,10 +5810,10 @@
     </row>
     <row r="61" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>76</v>
@@ -5809,13 +5822,13 @@
         <v>77</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H61" s="8" t="s">
         <v>402</v>
@@ -5841,7 +5854,7 @@
         <v>404</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>76</v>
@@ -5850,19 +5863,19 @@
         <v>77</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F62" s="13" t="s">
-        <v>175</v>
+        <v>216</v>
+      </c>
+      <c r="F62" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>394</v>
+        <v>405</v>
       </c>
       <c r="H62" s="8" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J62" s="11" t="s">
         <v>162</v>
@@ -5879,10 +5892,10 @@
     </row>
     <row r="63" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>76</v>
@@ -5897,13 +5910,13 @@
         <v>175</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>162</v>
@@ -5920,10 +5933,10 @@
     </row>
     <row r="64" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>76</v>
@@ -5938,7 +5951,7 @@
         <v>175</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>411</v>
+        <v>398</v>
       </c>
       <c r="H64" s="8" t="s">
         <v>412</v>
@@ -5964,7 +5977,7 @@
         <v>414</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>76</v>
@@ -6005,7 +6018,7 @@
         <v>418</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>76</v>
@@ -6014,10 +6027,10 @@
         <v>77</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="F66" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G66" s="8" t="s">
         <v>419</v>
@@ -6046,28 +6059,28 @@
         <v>422</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>76</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>250</v>
+        <v>423</v>
       </c>
       <c r="H67" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J67" s="11" t="s">
         <v>162</v>
@@ -6084,25 +6097,25 @@
     </row>
     <row r="68" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>84</v>
+        <v>397</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>157</v>
+        <v>317</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>426</v>
+        <v>250</v>
       </c>
       <c r="H68" s="8" t="s">
         <v>427</v>
@@ -6178,7 +6191,7 @@
         <v>85</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>158</v>
@@ -6219,10 +6232,10 @@
         <v>85</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F71" s="13" t="s">
-        <v>175</v>
+        <v>216</v>
+      </c>
+      <c r="F71" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G71" s="8" t="s">
         <v>438</v>
@@ -6301,10 +6314,10 @@
         <v>85</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="F73" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>446</v>
@@ -6339,10 +6352,10 @@
         <v>83</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>158</v>
@@ -6377,16 +6390,16 @@
         <v>84</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F75" s="13" t="s">
-        <v>190</v>
+        <v>317</v>
+      </c>
+      <c r="F75" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G75" s="8" t="s">
         <v>454</v>
@@ -6415,19 +6428,19 @@
         <v>457</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F76" s="10" t="s">
-        <v>158</v>
+      <c r="F76" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G76" s="8" t="s">
         <v>458</v>
@@ -6467,8 +6480,8 @@
       <c r="E77" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F77" s="13" t="s">
-        <v>175</v>
+      <c r="F77" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G77" s="8" t="s">
         <v>462</v>
@@ -6506,7 +6519,7 @@
         <v>64</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F78" s="13" t="s">
         <v>175</v>
@@ -6547,7 +6560,7 @@
         <v>64</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="F79" s="13" t="s">
         <v>175</v>
@@ -6585,13 +6598,13 @@
         <v>91</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="F80" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F80" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G80" s="8" t="s">
         <v>474</v>
@@ -6626,13 +6639,13 @@
         <v>91</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F81" s="13" t="s">
-        <v>190</v>
+        <v>317</v>
+      </c>
+      <c r="F81" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G81" s="8" t="s">
         <v>478</v>
@@ -6661,28 +6674,28 @@
         <v>481</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>482</v>
+        <v>92</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F82" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F82" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G82" s="8" t="s">
+        <v>482</v>
+      </c>
+      <c r="H82" s="8" t="s">
         <v>483</v>
       </c>
-      <c r="H82" s="8" t="s">
+      <c r="I82" s="8" t="s">
         <v>484</v>
-      </c>
-      <c r="I82" s="8" t="s">
-        <v>485</v>
       </c>
       <c r="J82" s="11" t="s">
         <v>162</v>
@@ -6699,10 +6712,10 @@
     </row>
     <row r="83" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="B83" s="8" t="s">
         <v>486</v>
-      </c>
-      <c r="B83" s="8" t="s">
-        <v>482</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>125</v>
@@ -6713,8 +6726,8 @@
       <c r="E83" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F83" s="13" t="s">
-        <v>175</v>
+      <c r="F83" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G83" s="8" t="s">
         <v>487</v>
@@ -6743,19 +6756,19 @@
         <v>490</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>156</v>
+        <v>64</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G84" s="8" t="s">
         <v>491</v>
@@ -6784,19 +6797,19 @@
         <v>494</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>126</v>
+        <v>486</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>44</v>
+        <v>156</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F85" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F85" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G85" s="8" t="s">
         <v>495</v>
@@ -6825,13 +6838,13 @@
         <v>498</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>499</v>
+        <v>126</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>157</v>
@@ -6840,13 +6853,13 @@
         <v>158</v>
       </c>
       <c r="G86" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="H86" s="8" t="s">
         <v>500</v>
       </c>
-      <c r="H86" s="8" t="s">
+      <c r="I86" s="8" t="s">
         <v>501</v>
-      </c>
-      <c r="I86" s="8" t="s">
-        <v>502</v>
       </c>
       <c r="J86" s="11" t="s">
         <v>162</v>
@@ -6863,10 +6876,10 @@
     </row>
     <row r="87" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="B87" s="8" t="s">
         <v>503</v>
-      </c>
-      <c r="B87" s="8" t="s">
-        <v>499</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>125</v>
@@ -6875,10 +6888,10 @@
         <v>101</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F87" s="13" t="s">
-        <v>175</v>
+        <v>157</v>
+      </c>
+      <c r="F87" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G87" s="8" t="s">
         <v>504</v>
@@ -6907,19 +6920,19 @@
         <v>507</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="D88" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F88" s="10" t="s">
-        <v>158</v>
+        <v>165</v>
+      </c>
+      <c r="F88" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G88" s="8" t="s">
         <v>508</v>
@@ -6948,7 +6961,7 @@
         <v>511</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>107</v>
@@ -6963,13 +6976,13 @@
         <v>158</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="H89" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J89" s="11" t="s">
         <v>162</v>
@@ -6986,13 +6999,13 @@
     </row>
     <row r="90" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="D90" s="8" t="s">
         <v>101</v>
@@ -7000,11 +7013,11 @@
       <c r="E90" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F90" s="13" t="s">
-        <v>175</v>
+      <c r="F90" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G90" s="8" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="H90" s="8" t="s">
         <v>516</v>
@@ -7030,10 +7043,10 @@
         <v>518</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>101</v>
@@ -7042,7 +7055,7 @@
         <v>157</v>
       </c>
       <c r="F91" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G91" s="8" t="s">
         <v>519</v>
@@ -7071,10 +7084,10 @@
         <v>522</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>101</v>
@@ -7112,10 +7125,10 @@
         <v>526</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>29</v>
+        <v>503</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>101</v>
@@ -7123,17 +7136,17 @@
       <c r="E93" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F93" s="10" t="s">
-        <v>158</v>
+      <c r="F93" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G93" s="8" t="s">
-        <v>237</v>
+        <v>527</v>
       </c>
       <c r="H93" s="8" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="I93" s="8" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="J93" s="11" t="s">
         <v>162</v>
@@ -7150,7 +7163,7 @@
     </row>
     <row r="94" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B94" s="8" t="s">
         <v>29</v>
@@ -7168,7 +7181,7 @@
         <v>158</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>530</v>
+        <v>237</v>
       </c>
       <c r="H94" s="8" t="s">
         <v>531</v>
@@ -7205,8 +7218,8 @@
       <c r="E95" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F95" s="13" t="s">
-        <v>175</v>
+      <c r="F95" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G95" s="8" t="s">
         <v>534</v>
@@ -7244,10 +7257,10 @@
         <v>101</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F96" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F96" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G96" s="8" t="s">
         <v>538</v>
@@ -7285,7 +7298,7 @@
         <v>101</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>158</v>
@@ -7328,8 +7341,8 @@
       <c r="E98" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F98" s="13" t="s">
-        <v>190</v>
+      <c r="F98" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G98" s="8" t="s">
         <v>546</v>
@@ -7361,7 +7374,7 @@
         <v>29</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>101</v>
@@ -7370,16 +7383,16 @@
         <v>157</v>
       </c>
       <c r="F99" s="13" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="G99" s="8" t="s">
-        <v>454</v>
+        <v>550</v>
       </c>
       <c r="H99" s="8" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="I99" s="8" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="J99" s="11" t="s">
         <v>162</v>
@@ -7396,7 +7409,7 @@
     </row>
     <row r="100" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="8" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B100" s="8" t="s">
         <v>29</v>
@@ -7408,19 +7421,19 @@
         <v>101</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F100" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="H100" s="8" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="I100" s="8" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>162</v>
@@ -7437,7 +7450,7 @@
     </row>
     <row r="101" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>29</v>
@@ -7449,13 +7462,13 @@
         <v>101</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="F101" s="13" t="s">
         <v>190</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>556</v>
+        <v>458</v>
       </c>
       <c r="H101" s="8" t="s">
         <v>557</v>
@@ -7484,25 +7497,25 @@
         <v>29</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D102" s="8" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="F102" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F102" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G102" s="8" t="s">
-        <v>250</v>
+        <v>560</v>
       </c>
       <c r="H102" s="8" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="I102" s="8" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>162</v>
@@ -7519,25 +7532,25 @@
     </row>
     <row r="103" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B103" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="F103" s="13" t="s">
-        <v>175</v>
+        <v>317</v>
+      </c>
+      <c r="F103" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>563</v>
+        <v>250</v>
       </c>
       <c r="H103" s="8" t="s">
         <v>564</v>
@@ -7572,10 +7585,10 @@
         <v>101</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F104" s="10" t="s">
-        <v>158</v>
+        <v>216</v>
+      </c>
+      <c r="F104" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G104" s="8" t="s">
         <v>567</v>
@@ -7604,28 +7617,28 @@
         <v>570</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>571</v>
+        <v>29</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D105" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G105" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="H105" s="8" t="s">
         <v>572</v>
       </c>
-      <c r="H105" s="8" t="s">
+      <c r="I105" s="8" t="s">
         <v>573</v>
-      </c>
-      <c r="I105" s="8" t="s">
-        <v>574</v>
       </c>
       <c r="J105" s="11" t="s">
         <v>162</v>
@@ -7642,10 +7655,10 @@
     </row>
     <row r="106" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="B106" s="8" t="s">
         <v>575</v>
-      </c>
-      <c r="B106" s="8" t="s">
-        <v>571</v>
       </c>
       <c r="C106" s="8" t="s">
         <v>112</v>
@@ -7656,8 +7669,8 @@
       <c r="E106" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F106" s="13" t="s">
-        <v>175</v>
+      <c r="F106" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G106" s="8" t="s">
         <v>576</v>
@@ -7686,7 +7699,7 @@
         <v>579</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C107" s="8" t="s">
         <v>112</v>
@@ -7695,10 +7708,10 @@
         <v>101</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F107" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F107" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G107" s="8" t="s">
         <v>580</v>
@@ -7727,16 +7740,16 @@
         <v>583</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D108" s="8" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="F108" s="10" t="s">
         <v>158</v>
@@ -7768,28 +7781,28 @@
         <v>587</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>119</v>
+        <v>575</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E109" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F109" s="13" t="s">
-        <v>175</v>
+      <c r="F109" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G109" s="8" t="s">
-        <v>121</v>
+        <v>588</v>
       </c>
       <c r="H109" s="8" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="I109" s="8" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="J109" s="11" t="s">
         <v>162</v>
@@ -7806,7 +7819,7 @@
     </row>
     <row r="110" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B110" s="8" t="s">
         <v>119</v>
@@ -7820,11 +7833,11 @@
       <c r="E110" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F110" s="10" t="s">
-        <v>158</v>
+      <c r="F110" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>591</v>
+        <v>121</v>
       </c>
       <c r="H110" s="8" t="s">
         <v>592</v>
@@ -7861,8 +7874,8 @@
       <c r="E111" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F111" s="13" t="s">
-        <v>175</v>
+      <c r="F111" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G111" s="8" t="s">
         <v>595</v>
@@ -7897,7 +7910,7 @@
         <v>118</v>
       </c>
       <c r="D112" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E112" s="8" t="s">
         <v>157</v>
@@ -7906,13 +7919,13 @@
         <v>175</v>
       </c>
       <c r="G112" s="8" t="s">
-        <v>220</v>
+        <v>599</v>
       </c>
       <c r="H112" s="8" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="I112" s="8" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="J112" s="11" t="s">
         <v>162</v>
@@ -7929,7 +7942,7 @@
     </row>
     <row r="113" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B113" s="8" t="s">
         <v>119</v>
@@ -7944,10 +7957,10 @@
         <v>157</v>
       </c>
       <c r="F113" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G113" s="8" t="s">
-        <v>602</v>
+        <v>220</v>
       </c>
       <c r="H113" s="8" t="s">
         <v>603</v>
@@ -7982,7 +7995,7 @@
         <v>156</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F114" s="13" t="s">
         <v>190</v>
@@ -8023,7 +8036,7 @@
         <v>156</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
       <c r="F115" s="13" t="s">
         <v>190</v>
@@ -8055,10 +8068,10 @@
         <v>613</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="D116" s="8" t="s">
         <v>156</v>
@@ -8096,28 +8109,28 @@
         <v>617</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>618</v>
+        <v>133</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E117" s="8" t="s">
         <v>157</v>
       </c>
       <c r="F117" s="13" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="G117" s="8" t="s">
+        <v>618</v>
+      </c>
+      <c r="H117" s="8" t="s">
         <v>619</v>
       </c>
-      <c r="H117" s="8" t="s">
+      <c r="I117" s="8" t="s">
         <v>620</v>
-      </c>
-      <c r="I117" s="8" t="s">
-        <v>621</v>
       </c>
       <c r="J117" s="11" t="s">
         <v>162</v>
@@ -8134,10 +8147,10 @@
     </row>
     <row r="118" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="B118" s="8" t="s">
         <v>622</v>
-      </c>
-      <c r="B118" s="8" t="s">
-        <v>618</v>
       </c>
       <c r="C118" s="8" t="s">
         <v>107</v>
@@ -8146,7 +8159,7 @@
         <v>101</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>313</v>
+        <v>157</v>
       </c>
       <c r="F118" s="13" t="s">
         <v>175</v>
@@ -8178,28 +8191,28 @@
         <v>626</v>
       </c>
       <c r="B119" s="8" t="s">
+        <v>622</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="F119" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="G119" s="8" t="s">
         <v>627</v>
       </c>
-      <c r="C119" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D119" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E119" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F119" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="G119" s="8" t="s">
+      <c r="H119" s="8" t="s">
         <v>628</v>
       </c>
-      <c r="H119" s="8" t="s">
+      <c r="I119" s="8" t="s">
         <v>629</v>
-      </c>
-      <c r="I119" s="8" t="s">
-        <v>630</v>
       </c>
       <c r="J119" s="11" t="s">
         <v>162</v>
@@ -8216,31 +8229,31 @@
     </row>
     <row r="120" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="B120" s="8" t="s">
         <v>631</v>
       </c>
-      <c r="B120" s="8" t="s">
-        <v>632</v>
-      </c>
       <c r="C120" s="8" t="s">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="D120" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E120" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F120" s="13" t="s">
-        <v>175</v>
+      <c r="F120" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G120" s="8" t="s">
+        <v>632</v>
+      </c>
+      <c r="H120" s="8" t="s">
         <v>633</v>
       </c>
-      <c r="H120" s="8" t="s">
+      <c r="I120" s="8" t="s">
         <v>634</v>
-      </c>
-      <c r="I120" s="8" t="s">
-        <v>635</v>
       </c>
       <c r="J120" s="11" t="s">
         <v>162</v>
@@ -8257,10 +8270,10 @@
     </row>
     <row r="121" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
+        <v>635</v>
+      </c>
+      <c r="B121" s="8" t="s">
         <v>636</v>
-      </c>
-      <c r="B121" s="8" t="s">
-        <v>632</v>
       </c>
       <c r="C121" s="8" t="s">
         <v>118</v>
@@ -8275,13 +8288,13 @@
         <v>175</v>
       </c>
       <c r="G121" s="8" t="s">
-        <v>491</v>
+        <v>637</v>
       </c>
       <c r="H121" s="8" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="I121" s="8" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="J121" s="11" t="s">
         <v>162</v>
@@ -8298,25 +8311,25 @@
     </row>
     <row r="122" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>170</v>
+        <v>636</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="D122" s="8" t="s">
         <v>156</v>
       </c>
       <c r="E122" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F122" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F122" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G122" s="8" t="s">
-        <v>640</v>
+        <v>495</v>
       </c>
       <c r="H122" s="8" t="s">
         <v>641</v>
@@ -8357,13 +8370,13 @@
         <v>158</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>121</v>
+        <v>644</v>
       </c>
       <c r="H123" s="8" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="I123" s="8" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="J123" s="11" t="s">
         <v>162</v>
@@ -8380,7 +8393,7 @@
     </row>
     <row r="124" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="8" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B124" s="8" t="s">
         <v>170</v>
@@ -8394,11 +8407,11 @@
       <c r="E124" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F124" s="13" t="s">
-        <v>175</v>
+      <c r="F124" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>647</v>
+        <v>121</v>
       </c>
       <c r="H124" s="8" t="s">
         <v>648</v>
@@ -8465,28 +8478,28 @@
         <v>654</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>137</v>
+        <v>28</v>
       </c>
       <c r="D126" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E126" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F126" s="10" t="s">
-        <v>158</v>
+        <v>170</v>
+      </c>
+      <c r="F126" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G126" s="8" t="s">
-        <v>141</v>
+        <v>655</v>
       </c>
       <c r="H126" s="8" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="I126" s="8" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="J126" s="11" t="s">
         <v>162</v>
@@ -8503,7 +8516,7 @@
     </row>
     <row r="127" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B127" s="8" t="s">
         <v>138</v>
@@ -8524,10 +8537,10 @@
         <v>141</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="I127" s="8" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="J127" s="11" t="s">
         <v>162</v>
@@ -8544,7 +8557,7 @@
     </row>
     <row r="128" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B128" s="8" t="s">
         <v>138</v>
@@ -8558,17 +8571,17 @@
       <c r="E128" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F128" s="13" t="s">
-        <v>175</v>
+      <c r="F128" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G128" s="8" t="s">
         <v>141</v>
       </c>
       <c r="H128" s="8" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="I128" s="8" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="J128" s="11" t="s">
         <v>162</v>
@@ -8585,7 +8598,7 @@
     </row>
     <row r="129" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B129" s="8" t="s">
         <v>138</v>
@@ -8599,11 +8612,11 @@
       <c r="E129" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F129" s="10" t="s">
-        <v>158</v>
+      <c r="F129" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G129" s="8" t="s">
-        <v>664</v>
+        <v>141</v>
       </c>
       <c r="H129" s="8" t="s">
         <v>665</v>
@@ -8624,9 +8637,50 @@
         <v>1</v>
       </c>
     </row>
+    <row r="130" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="8" t="s">
+        <v>667</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D130" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E130" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F130" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G130" s="8" t="s">
+        <v>668</v>
+      </c>
+      <c r="H130" s="8" t="s">
+        <v>669</v>
+      </c>
+      <c r="I130" s="8" t="s">
+        <v>670</v>
+      </c>
+      <c r="J130" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="K130" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="L130" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="M130" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M129"/>
-  <conditionalFormatting sqref="J2:J129">
+  <autoFilter ref="A1:M130"/>
+  <conditionalFormatting sqref="J2:J130">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -8638,10 +8692,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="J10:J129">
+    <dataValidation type="list" sqref="J10:J130">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J129">
+    <dataValidation type="list" sqref="J2:J130">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8662,7 +8716,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>1</v>
@@ -8688,22 +8742,22 @@
         <v>21</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8711,23 +8765,23 @@
         <v>155</v>
       </c>
       <c r="B3" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A3)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A3)</f>
         <v>10</v>
       </c>
       <c r="C3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A3,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>10</v>
       </c>
       <c r="G3" s="16">
@@ -8740,23 +8794,23 @@
         <v>201</v>
       </c>
       <c r="B4" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A4)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A4)</f>
         <v>7</v>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A4,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G4" s="16">
@@ -8769,23 +8823,23 @@
         <v>228</v>
       </c>
       <c r="B5" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A5)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A5)</f>
         <v>1</v>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A5,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G5" s="16">
@@ -8798,23 +8852,23 @@
         <v>233</v>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A6)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A6)</f>
         <v>4</v>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A6,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G6" s="16">
@@ -8827,24 +8881,24 @@
         <v>249</v>
       </c>
       <c r="B7" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A7)</f>
-        <v>7</v>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A7)</f>
+        <v>8</v>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A7,'Test cases'!$J$2:$J$129,"Not run")</f>
-        <v>7</v>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <v>8</v>
       </c>
       <c r="G7" s="16">
         <f>IF(B7=0,0,C7/B7)</f>
@@ -8853,26 +8907,26 @@
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B8" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A8)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A8,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G8" s="16">
@@ -8882,26 +8936,26 @@
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B9" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A9)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A9)</f>
         <v>4</v>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A9,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G9" s="16">
@@ -8914,23 +8968,23 @@
         <v>43</v>
       </c>
       <c r="B10" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A10)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A10)</f>
         <v>4</v>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A10,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G10" s="16">
@@ -8940,26 +8994,26 @@
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B11" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A11)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A11)</f>
         <v>2</v>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A11,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G11" s="16">
@@ -8969,26 +9023,26 @@
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B12" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A12)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A12)</f>
         <v>1</v>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A12,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G12" s="16">
@@ -8998,26 +9052,26 @@
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B13" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A13)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A13)</f>
         <v>5</v>
       </c>
       <c r="C13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A13,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>5</v>
       </c>
       <c r="G13" s="16">
@@ -9027,26 +9081,26 @@
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B14" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A14)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A14)</f>
         <v>8</v>
       </c>
       <c r="C14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A14,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G14" s="16">
@@ -9056,26 +9110,26 @@
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B15" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A15)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A15)</f>
         <v>9</v>
       </c>
       <c r="C15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A15,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>9</v>
       </c>
       <c r="G15" s="16">
@@ -9088,23 +9142,23 @@
         <v>84</v>
       </c>
       <c r="B16" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A16)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A16)</f>
         <v>8</v>
       </c>
       <c r="C16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A16,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G16" s="16">
@@ -9117,23 +9171,23 @@
         <v>92</v>
       </c>
       <c r="B17" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A17)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A17)</f>
         <v>6</v>
       </c>
       <c r="C17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A17,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>6</v>
       </c>
       <c r="G17" s="16">
@@ -9143,26 +9197,26 @@
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="B18" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A18)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A18)</f>
         <v>3</v>
       </c>
       <c r="C18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A18,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G18" s="16">
@@ -9175,23 +9229,23 @@
         <v>126</v>
       </c>
       <c r="B19" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A19)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A19,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G19" s="16">
@@ -9201,26 +9255,26 @@
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="B20" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A20)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A20)</f>
         <v>7</v>
       </c>
       <c r="C20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A20,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G20" s="16">
@@ -9233,23 +9287,23 @@
         <v>29</v>
       </c>
       <c r="B21" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A21)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A21)</f>
         <v>12</v>
       </c>
       <c r="C21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A21,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>12</v>
       </c>
       <c r="G21" s="16">
@@ -9259,26 +9313,26 @@
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B22" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A22)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A22)</f>
         <v>4</v>
       </c>
       <c r="C22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A22,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G22" s="16">
@@ -9291,23 +9345,23 @@
         <v>119</v>
       </c>
       <c r="B23" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A23)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A23)</f>
         <v>7</v>
       </c>
       <c r="C23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A23,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G23" s="16">
@@ -9320,23 +9374,23 @@
         <v>133</v>
       </c>
       <c r="B24" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A24)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A24)</f>
         <v>1</v>
       </c>
       <c r="C24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A24,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G24" s="16">
@@ -9346,26 +9400,26 @@
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="B25" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A25)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A25)</f>
         <v>2</v>
       </c>
       <c r="C25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A25,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G25" s="16">
@@ -9375,26 +9429,26 @@
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B26" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A26)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A26,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="16">
@@ -9404,26 +9458,26 @@
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="B27" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A27)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A27)</f>
         <v>2</v>
       </c>
       <c r="C27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A27,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G27" s="16">
@@ -9436,23 +9490,23 @@
         <v>170</v>
       </c>
       <c r="B28" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A28)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A28)</f>
         <v>4</v>
       </c>
       <c r="C28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A28,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G28" s="16">
@@ -9465,23 +9519,23 @@
         <v>138</v>
       </c>
       <c r="B29" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$129,$A29)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$130,$A29)</f>
         <v>4</v>
       </c>
       <c r="C29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$129,$A29,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G29" s="16">
@@ -9491,11 +9545,11 @@
     </row>
     <row r="30" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="B30" s="18">
         <f>SUM(B3:B29)</f>
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" s="18">
         <f>SUM(C3:C29)</f>
@@ -9511,7 +9565,7 @@
       </c>
       <c r="F30" s="18">
         <f>SUM(F3:F29)</f>
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G30" s="19">
         <f>IF(B30=0,0,C30/B30)</f>
@@ -9520,7 +9574,7 @@
     </row>
     <row r="32" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>1</v>
@@ -9546,22 +9600,22 @@
         <v>12</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -9569,23 +9623,23 @@
         <v>158</v>
       </c>
       <c r="B34" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$129,A34)</f>
+        <f>COUNTIF('Test cases'!$F$2:$F$130,A34)</f>
         <v>64</v>
       </c>
       <c r="C34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A34,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>64</v>
       </c>
       <c r="G34" s="22">
@@ -9598,24 +9652,24 @@
         <v>175</v>
       </c>
       <c r="B35" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$129,A35)</f>
-        <v>46</v>
+        <f>COUNTIF('Test cases'!$F$2:$F$130,A35)</f>
+        <v>47</v>
       </c>
       <c r="C35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A35,'Test cases'!$J$2:$J$129,"Not run")</f>
-        <v>46</v>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <v>47</v>
       </c>
       <c r="G35" s="22">
         <f>IF(B35=0,0,C35/B35)</f>
@@ -9627,23 +9681,23 @@
         <v>190</v>
       </c>
       <c r="B36" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$129,A36)</f>
+        <f>COUNTIF('Test cases'!$F$2:$F$130,A36)</f>
         <v>18</v>
       </c>
       <c r="C36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$129,$A36,'Test cases'!$J$2:$J$129,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Not run")</f>
         <v>18</v>
       </c>
       <c r="G36" s="22">
@@ -9653,7 +9707,7 @@
     </row>
     <row r="38" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
   </sheetData>
@@ -9676,19 +9730,19 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9696,16 +9750,16 @@
         <v>44</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9713,16 +9767,16 @@
         <v>64</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9730,16 +9784,16 @@
         <v>77</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9747,16 +9801,16 @@
         <v>85</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9764,21 +9818,21 @@
         <v>101</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjust page on a phone: a swipe scrolls the window from anywhere (it used to be trapped by the photo and the page preview); the corner dots, pinching and a zoomed-in picture still keep their touch; real-touch test and workbook row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/REIMSYS-test-cases.xlsx
+++ b/docs/REIMSYS-test-cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1945" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1958" uniqueCount="705">
   <si>
     <t>REIMSYS: use cases and test cases</t>
   </si>
@@ -949,6 +949,20 @@
     <t>TC-036</t>
   </si>
   <si>
+    <t>A phone; the scan editor (Adjust page) is open with a tall photo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Scroll down past the photo to the page preview and the buttons.
+2. Starting a swipe ON the saved-page preview, scroll back up. Then start a swipe on the photo and scroll down.
+3. Drag a corner dot; pinch the preview; drag a zoomed-in preview; press Fit and swipe again.</t>
+  </si>
+  <si>
+    <t>Every swipe scrolls the window, wherever it starts (the preview, the photo, the buttons). Only a corner dot, a pinch and a zoomed-in picture keep the touch: the dot moves, the preview zooms, the zoomed picture pans. After Fit, swiping scrolls the window again.</t>
+  </si>
+  <si>
+    <t>TC-037</t>
+  </si>
+  <si>
     <t>A white receipt on a light desk.</t>
   </si>
   <si>
@@ -958,7 +972,7 @@
     <t>The receipt is outlined when it is clearly lighter than the desk; otherwise the corners start on the whole photo and can be dragged.</t>
   </si>
   <si>
-    <t>TC-037</t>
+    <t>TC-038</t>
   </si>
   <si>
     <t>The scan editor is open.</t>
@@ -970,7 +984,7 @@
     <t>All text is readable (nothing white on white), including when opened over the live camera screen.</t>
   </si>
   <si>
-    <t>TC-038</t>
+    <t>TC-039</t>
   </si>
   <si>
     <t>A phone.</t>
@@ -982,7 +996,7 @@
     <t>The date box is as wide as the other boxes and stays inside the card; the page does not scroll sideways.</t>
   </si>
   <si>
-    <t>TC-039</t>
+    <t>TC-040</t>
   </si>
   <si>
     <t>A Submitted receipt that nobody has opened yet.</t>
@@ -995,7 +1009,7 @@
     <t>The receipt goes back to Draft and leaves the Checker's queue. It can be edited and submitted again.</t>
   </si>
   <si>
-    <t>TC-040</t>
+    <t>TC-041</t>
   </si>
   <si>
     <t>Permission</t>
@@ -1010,7 +1024,7 @@
     <t>It is refused. A Med Ref can only see their own receipts.</t>
   </si>
   <si>
-    <t>TC-041</t>
+    <t>TC-042</t>
   </si>
   <si>
     <t>A receipt that is Checked or later.</t>
@@ -1022,7 +1036,7 @@
     <t>Editing is not offered (and the server refuses it). A paid receipt cannot be edited, withdrawn or deleted.</t>
   </si>
   <si>
-    <t>TC-042</t>
+    <t>TC-043</t>
   </si>
   <si>
     <t>The same receipt open in two windows.</t>
@@ -1035,7 +1049,7 @@
     <t>Window B is told the receipt changed and does not overwrite it (stale edits are refused).</t>
   </si>
   <si>
-    <t>TC-043</t>
+    <t>TC-044</t>
   </si>
   <si>
     <t>Import</t>
@@ -1052,7 +1066,7 @@
     <t>The preview lists each row and the error for the bad one. Only the valid rows are saved as Drafts. The bad row is not saved.</t>
   </si>
   <si>
-    <t>TC-044</t>
+    <t>TC-045</t>
   </si>
   <si>
     <t>On Import.</t>
@@ -1064,7 +1078,7 @@
     <t>It is refused with a clear message.</t>
   </si>
   <si>
-    <t>TC-045</t>
+    <t>TC-046</t>
   </si>
   <si>
     <t>Export</t>
@@ -1080,7 +1094,7 @@
     <t>The file contains the receipts the person may see, with invoice, VAT and withholding columns, and no category column.</t>
   </si>
   <si>
-    <t>TC-046</t>
+    <t>TC-047</t>
   </si>
   <si>
     <t>Receipt list</t>
@@ -1096,7 +1110,7 @@
     <t>The list and the counts on the status buttons follow every filter. Clear filters returns to everything.</t>
   </si>
   <si>
-    <t>TC-047</t>
+    <t>TC-048</t>
   </si>
   <si>
     <t>Several pages of receipts.</t>
@@ -1109,7 +1123,7 @@
     <t>The footer total is the amount of ALL matching receipts (every page), and changes with the filters. It equals the sum of the rows over all pages.</t>
   </si>
   <si>
-    <t>TC-048</t>
+    <t>TC-049</t>
   </si>
   <si>
     <t>Two Med Refs have receipts.</t>
@@ -1121,7 +1135,7 @@
     <t>Each sees only their own receipts and their own total.</t>
   </si>
   <si>
-    <t>TC-049</t>
+    <t>TC-050</t>
   </si>
   <si>
     <t xml:space="preserve">1. Open My receipts.
@@ -1131,7 +1145,7 @@
     <t>The search stays visible; the filters open and close behind a Filters button; status buttons scroll sideways in one row.</t>
   </si>
   <si>
-    <t>TC-050</t>
+    <t>TC-051</t>
   </si>
   <si>
     <t>A computer window at least 780 px tall.</t>
@@ -1143,7 +1157,7 @@
     <t>The page and menu stay still; only the rows scroll; column titles stay pinned; the footer stays at the bottom.</t>
   </si>
   <si>
-    <t>TC-051</t>
+    <t>TC-052</t>
   </si>
   <si>
     <t>Check</t>
@@ -1160,7 +1174,7 @@
     <t>Before the evidence is opened the buttons are locked with an explanation. Opening it is recorded. After opening, Mark checked works and the receipt becomes Checked; the Approver is told.</t>
   </si>
   <si>
-    <t>TC-052</t>
+    <t>TC-053</t>
   </si>
   <si>
     <t>A Submitted receipt.</t>
@@ -1175,7 +1189,7 @@
     <t>The receipt is Returned. The Med Ref gets a notice and an email that name the ticked problems and the note.</t>
   </si>
   <si>
-    <t>TC-053</t>
+    <t>TC-054</t>
   </si>
   <si>
     <t>The Return window is open.</t>
@@ -1188,7 +1202,7 @@
     <t>Both are refused: a problem or words are required.</t>
   </si>
   <si>
-    <t>TC-054</t>
+    <t>TC-055</t>
   </si>
   <si>
     <t>A Returned receipt with ticked problems.</t>
@@ -1202,7 +1216,7 @@
     <t>Fix opens the form on the right step. After submitting, the receipt is Submitted again and the ticked problems are cleared.</t>
   </si>
   <si>
-    <t>TC-055</t>
+    <t>TC-056</t>
   </si>
   <si>
     <t>The Checker has their own Submitted receipt (via another role).</t>
@@ -1214,7 +1228,7 @@
     <t>It is refused: reviewers cannot review their own receipts.</t>
   </si>
   <si>
-    <t>TC-056</t>
+    <t>TC-057</t>
   </si>
   <si>
     <t>A receipt open to the Checker.</t>
@@ -1227,7 +1241,7 @@
     <t>The comment appears on the receipt for both, with the author and time, and the other person gets a notice.</t>
   </si>
   <si>
-    <t>TC-057</t>
+    <t>TC-058</t>
   </si>
   <si>
     <t>Five Submitted receipts; evidence opened on three.</t>
@@ -1240,7 +1254,7 @@
     <t>The three are Checked. The other two are skipped and listed with the reason. At most 25 can be selected.</t>
   </si>
   <si>
-    <t>TC-058</t>
+    <t>TC-059</t>
   </si>
   <si>
     <t>A receipt that has waited several days.</t>
@@ -1252,7 +1266,7 @@
     <t>The waiting time shows (e.g. "6 days ago") and is highlighted when it passes the reminder limit.</t>
   </si>
   <si>
-    <t>TC-059</t>
+    <t>TC-060</t>
   </si>
   <si>
     <t>Decision</t>
@@ -1268,7 +1282,7 @@
     <t>The receipt is Approved, a reimbursement document (REIM-yyyy-nnnnnn) is created and can be downloaded and printed, and the Med Ref and Accounting are told.</t>
   </si>
   <si>
-    <t>TC-060</t>
+    <t>TC-061</t>
   </si>
   <si>
     <t>1. Press Disapprove and give a reason; confirm.</t>
@@ -1277,7 +1291,7 @@
     <t>The receipt is Disapproved with the reason shown to the Med Ref. Disapproved is final.</t>
   </si>
   <si>
-    <t>TC-061</t>
+    <t>TC-062</t>
   </si>
   <si>
     <t>The Disapprove or Reserve window is open.</t>
@@ -1289,7 +1303,7 @@
     <t>A reason (Disapprove) or a note (Reserve) is required.</t>
   </si>
   <si>
-    <t>TC-062</t>
+    <t>TC-063</t>
   </si>
   <si>
     <t xml:space="preserve">1. Press Reserve with a note.
@@ -1299,7 +1313,7 @@
     <t>It becomes Reserved (on hold) and the Med Ref is told; after Release it is back in the approval queue.</t>
   </si>
   <si>
-    <t>TC-063</t>
+    <t>TC-064</t>
   </si>
   <si>
     <t>1. Press Ask for more proof.</t>
@@ -1308,7 +1322,7 @@
     <t>The receipt goes back to the Med Ref, who can add proof and submit; it is then checked from the start.</t>
   </si>
   <si>
-    <t>TC-064</t>
+    <t>TC-065</t>
   </si>
   <si>
     <t>An Approved, unpaid receipt, within the undo time.</t>
@@ -1320,7 +1334,7 @@
     <t>It returns to Checked and the Med Ref is told to disregard the earlier approval. After the undo time (Access &gt; Settings) the button is gone.</t>
   </si>
   <si>
-    <t>TC-065</t>
+    <t>TC-066</t>
   </si>
   <si>
     <t>Several Checked receipts opened by the Approver.</t>
@@ -1332,7 +1346,7 @@
     <t>The ready ones are Approved with their documents. Any not ready are skipped with a reason.</t>
   </si>
   <si>
-    <t>TC-066</t>
+    <t>TC-067</t>
   </si>
   <si>
     <t>A Submitted (not yet Checked) receipt.</t>
@@ -1344,7 +1358,7 @@
     <t>The Approver cannot see or decide it: only checked receipts reach them.</t>
   </si>
   <si>
-    <t>TC-067</t>
+    <t>TC-068</t>
   </si>
   <si>
     <t>1. Try to approve a receipt by address or from the API.</t>
@@ -1353,7 +1367,7 @@
     <t>It is refused (no review rights).</t>
   </si>
   <si>
-    <t>TC-068</t>
+    <t>TC-069</t>
   </si>
   <si>
     <t>Approved receipts for two people.</t>
@@ -1365,7 +1379,7 @@
     <t>Receipts are grouped by person with the count and total; a header stays visible while scrolling; a footer shows people, receipts and total to pay.</t>
   </si>
   <si>
-    <t>TC-069</t>
+    <t>TC-070</t>
   </si>
   <si>
     <t>Approved receipts for one person.</t>
@@ -1380,7 +1394,7 @@
     <t>A payment number (PAY-yyyy-nnnnnn) is created. The receipts become Paid, show the payment card and cannot be edited. The Med Ref is emailed.</t>
   </si>
   <si>
-    <t>TC-070</t>
+    <t>TC-071</t>
   </si>
   <si>
     <t>The payment window is open.</t>
@@ -1392,7 +1406,7 @@
     <t>Each is refused with a clear message. A shortfall needs a reason. One payment covers one person only (up to 25 receipts).</t>
   </si>
   <si>
-    <t>TC-071</t>
+    <t>TC-072</t>
   </si>
   <si>
     <t>A Paid receipt.</t>
@@ -1404,7 +1418,7 @@
     <t>The receipt returns to Approved, the Med Ref is told, and the original payment record stays (it is never deleted).</t>
   </si>
   <si>
-    <t>TC-072</t>
+    <t>TC-073</t>
   </si>
   <si>
     <t>Paid receipts in a period.</t>
@@ -1416,7 +1430,7 @@
     <t>One row per paid receipt with the payment date, method and amounts.</t>
   </si>
   <si>
-    <t>TC-073</t>
+    <t>TC-074</t>
   </si>
   <si>
     <t>Signed in as Checker, Approver or Med Ref.</t>
@@ -1428,7 +1442,7 @@
     <t>The screen is not offered and the server refuses.</t>
   </si>
   <si>
-    <t>TC-074</t>
+    <t>TC-075</t>
   </si>
   <si>
     <t>Default rights.</t>
@@ -1440,7 +1454,7 @@
     <t>None of them are available to the Super Admin by default, so one person cannot run the whole chain.</t>
   </si>
   <si>
-    <t>TC-075</t>
+    <t>TC-076</t>
   </si>
   <si>
     <t>Access &gt; Settings.</t>
@@ -1452,7 +1466,7 @@
     <t>The methods are offered in the payment window. At most 12 methods; empty names refused.</t>
   </si>
   <si>
-    <t>TC-076</t>
+    <t>TC-077</t>
   </si>
   <si>
     <t>Approved receipts in the month.</t>
@@ -1467,7 +1481,7 @@
     <t>The count and total match the Approved (and Paid) receipts in the range. The report opens in the viewer with totals, by-type breakdown and the record table.</t>
   </si>
   <si>
-    <t>TC-077</t>
+    <t>TC-078</t>
   </si>
   <si>
     <t>A report exists.</t>
@@ -1479,7 +1493,7 @@
     <t>All three open and carry the same records and totals.</t>
   </si>
   <si>
-    <t>TC-078</t>
+    <t>TC-079</t>
   </si>
   <si>
     <t>On Reports.</t>
@@ -1491,7 +1505,7 @@
     <t>The first shows "Choose a valid date range"; the second disables Generate.</t>
   </si>
   <si>
-    <t>TC-079</t>
+    <t>TC-080</t>
   </si>
   <si>
     <t>Approved receipts for several people and types.</t>
@@ -1503,7 +1517,7 @@
     <t>Only matching records appear; pending, returned and disapproved receipts are never included.</t>
   </si>
   <si>
-    <t>TC-080</t>
+    <t>TC-081</t>
   </si>
   <si>
     <t>Two people made reports.</t>
@@ -1515,7 +1529,7 @@
     <t>A person sees only reports they made (an administrator may see more).</t>
   </si>
   <si>
-    <t>TC-081</t>
+    <t>TC-082</t>
   </si>
   <si>
     <t>A report with many rows.</t>
@@ -1527,7 +1541,7 @@
     <t>Column titles, the first column and the Total row stay in view; the page does not scroll.</t>
   </si>
   <si>
-    <t>TC-082</t>
+    <t>TC-083</t>
   </si>
   <si>
     <t>Dashboard</t>
@@ -1542,7 +1556,7 @@
     <t>Each role sees its own tiles and queue (Checker: To check; Approver: To decide; Accounting: To pay; Med Ref: Needs your action; Super Admin: Waiting for review). The highlighted first tile is the queue.</t>
   </si>
   <si>
-    <t>TC-083</t>
+    <t>TC-084</t>
   </si>
   <si>
     <t>Receipts in several statuses.</t>
@@ -1554,7 +1568,7 @@
     <t>The Receipts list opens already filtered to that status.</t>
   </si>
   <si>
-    <t>TC-084</t>
+    <t>TC-085</t>
   </si>
   <si>
     <t>A computer.</t>
@@ -1566,7 +1580,7 @@
     <t>It fits the window: the queue and Recent activity scroll inside their cards; the greeting is one line.</t>
   </si>
   <si>
-    <t>TC-085</t>
+    <t>TC-086</t>
   </si>
   <si>
     <t>A Med Ref with a receipt in review.</t>
@@ -1579,7 +1593,7 @@
     <t>The bell count increases; the notice names the receipt and opens it.</t>
   </si>
   <si>
-    <t>TC-086</t>
+    <t>TC-087</t>
   </si>
   <si>
     <t>Email</t>
@@ -1595,7 +1609,7 @@
     <t>One email arrives for each event with the right wording and a link button (https servers). Each shows status "sent" with the mail server's answer.</t>
   </si>
   <si>
-    <t>TC-087</t>
+    <t>TC-088</t>
   </si>
   <si>
     <t>Demo accounts on example.com.</t>
@@ -1607,7 +1621,7 @@
     <t>Nothing is sent. The Email log shows "logged" with "Example address, not a real mailbox".</t>
   </si>
   <si>
-    <t>TC-088</t>
+    <t>TC-089</t>
   </si>
   <si>
     <t>Access &gt; Email.</t>
@@ -1620,7 +1634,7 @@
     <t>Test connection reports success without sending. The test email arrives and shows "sent".</t>
   </si>
   <si>
-    <t>TC-089</t>
+    <t>TC-090</t>
   </si>
   <si>
     <t>1. Press Run full check.</t>
@@ -1629,7 +1643,7 @@
     <t>Five steps are listed (account, password key, server name, ports, login) each with a tick or a cross and, for a failure, what to do. Nothing is sent. Running it is in the audit log.</t>
   </si>
   <si>
-    <t>TC-090</t>
+    <t>TC-091</t>
   </si>
   <si>
     <t>A failed email in the log.</t>
@@ -1641,7 +1655,7 @@
     <t>It is queued again and its status updates.</t>
   </si>
   <si>
-    <t>TC-091</t>
+    <t>TC-092</t>
   </si>
   <si>
     <t>Receipts waiting several days.</t>
@@ -1653,7 +1667,7 @@
     <t>The Checker, Approver, Accounting and Med Ref get reminders only for what is waiting longer than the days set; a receipt that has not waited long gets none.</t>
   </si>
   <si>
-    <t>TC-092</t>
+    <t>TC-093</t>
   </si>
   <si>
     <t>Access &gt; Email templates.</t>
@@ -1665,7 +1679,7 @@
     <t>The change shows in the sample; unknown placeholders are refused.</t>
   </si>
   <si>
-    <t>TC-093</t>
+    <t>TC-094</t>
   </si>
   <si>
     <t xml:space="preserve">1. Access &gt; Users &gt; Add user (name, email, role).
@@ -1675,7 +1689,7 @@
     <t>The user appears in the list as Invited. They can sign in with the temporary password and must choose their own.</t>
   </si>
   <si>
-    <t>TC-094</t>
+    <t>TC-095</t>
   </si>
   <si>
     <t>A user with receipts.</t>
@@ -1688,7 +1702,7 @@
     <t>The user is signed out at once and cannot sign in; their receipts and history stay. They can be switched on again.</t>
   </si>
   <si>
-    <t>TC-095</t>
+    <t>TC-096</t>
   </si>
   <si>
     <t>A locked or forgotten account.</t>
@@ -1700,7 +1714,7 @@
     <t>A new temporary password is shown once and other sessions end; Unlock lets the person try again. Both are in the audit log.</t>
   </si>
   <si>
-    <t>TC-096</t>
+    <t>TC-097</t>
   </si>
   <si>
     <t>One active Super Admin only.</t>
@@ -1712,7 +1726,7 @@
     <t>It is refused: there must always be an active administrator.</t>
   </si>
   <si>
-    <t>TC-097</t>
+    <t>TC-098</t>
   </si>
   <si>
     <t>Roles and permissions tab.</t>
@@ -1725,7 +1739,7 @@
     <t>The change applies on their next action and is in the audit log. Locked rights (check, approve, pay, manage users/roles/settings) cannot be unticked.</t>
   </si>
   <si>
-    <t>TC-098</t>
+    <t>TC-099</t>
   </si>
   <si>
     <t>Roles tab.</t>
@@ -1737,7 +1751,7 @@
     <t>The role can be given to users and they see only what it allows (menu and Help guides follow the rights).</t>
   </si>
   <si>
-    <t>TC-099</t>
+    <t>TC-100</t>
   </si>
   <si>
     <t xml:space="preserve">1. Change a form rule (for example turn off "Accept receipts without a BIR invoice") and Save.
@@ -1747,7 +1761,7 @@
     <t>The "No" answer is no longer offered. Reset everything to default restores the starting values.</t>
   </si>
   <si>
-    <t>TC-100</t>
+    <t>TC-101</t>
   </si>
   <si>
     <t>1. Enter a value outside the allowed range (for example 0 for the undo time).</t>
@@ -1756,7 +1770,7 @@
     <t>The box shows an error; Save stays off.</t>
   </si>
   <si>
-    <t>TC-101</t>
+    <t>TC-102</t>
   </si>
   <si>
     <t>Access &gt; Company.</t>
@@ -1768,7 +1782,7 @@
     <t>They appear on documents, reports and emails.</t>
   </si>
   <si>
-    <t>TC-102</t>
+    <t>TC-103</t>
   </si>
   <si>
     <t>1. Open /access and /audit by address.</t>
@@ -1777,7 +1791,7 @@
     <t>Both send the person back to the Dashboard.</t>
   </si>
   <si>
-    <t>TC-103</t>
+    <t>TC-104</t>
   </si>
   <si>
     <t>Access &gt; Settings (and any number box in the app).</t>
@@ -1790,7 +1804,7 @@
     <t>Only digits are accepted ( and the decimal point where decimals make sense). The letters e/E and the signs + and - cannot be typed or pasted. Whole-number boxes ignore the point.</t>
   </si>
   <si>
-    <t>TC-104</t>
+    <t>TC-105</t>
   </si>
   <si>
     <t>The web app is newer than the API (for example the API was not restarted after an update).</t>
@@ -1803,7 +1817,7 @@
     <t>A red message says the page is newer than the server and lists the settings the server does not know. Those settings are hidden (no empty "Required" boxes), the other settings still change and save, and nothing is silently dropped. After the API is rebuilt and restarted the message is gone and every setting shows and saves.</t>
   </si>
   <si>
-    <t>TC-105</t>
+    <t>TC-106</t>
   </si>
   <si>
     <t>Audit log</t>
@@ -1818,7 +1832,7 @@
     <t>Entries show who, what, when and (where relevant) the old and new values. Filters work together.</t>
   </si>
   <si>
-    <t>TC-106</t>
+    <t>TC-107</t>
   </si>
   <si>
     <t>Audit log open.</t>
@@ -1830,7 +1844,7 @@
     <t>A CSV with the filtered entries downloads.</t>
   </si>
   <si>
-    <t>TC-107</t>
+    <t>TC-108</t>
   </si>
   <si>
     <t>Access to the database server.</t>
@@ -1842,7 +1856,7 @@
     <t>The database refuses. The app can only read and add entries.</t>
   </si>
   <si>
-    <t>TC-108</t>
+    <t>TC-109</t>
   </si>
   <si>
     <t>A Checker opens evidence.</t>
@@ -1855,7 +1869,7 @@
     <t>Each view, download and print is recorded with the person and time.</t>
   </si>
   <si>
-    <t>TC-109</t>
+    <t>TC-110</t>
   </si>
   <si>
     <t>1. Profile &gt; Details: change name, phone, branch; Save.</t>
@@ -1864,7 +1878,7 @@
     <t>A message confirms; the new name shows in the side menu; a one-letter name is refused. The email cannot be changed here.</t>
   </si>
   <si>
-    <t>TC-110</t>
+    <t>TC-111</t>
   </si>
   <si>
     <t>Profile open.</t>
@@ -1876,7 +1890,7 @@
     <t>The photo is cropped square and shrunk, then accepted; the side menu and top bar show it at once.</t>
   </si>
   <si>
-    <t>TC-111</t>
+    <t>TC-112</t>
   </si>
   <si>
     <t>A profile photo exists.</t>
@@ -1889,7 +1903,7 @@
     <t>The new picture shows everywhere straight away. After Remove photo the initials come back and the button says Add photo; it is in the audit log.</t>
   </si>
   <si>
-    <t>TC-112</t>
+    <t>TC-113</t>
   </si>
   <si>
     <t xml:space="preserve">1. Profile &gt; Security: look at Where you are signed in.
@@ -1899,7 +1913,7 @@
     <t>This device is marked "This device". The other device is signed out.</t>
   </si>
   <si>
-    <t>TC-113</t>
+    <t>TC-114</t>
   </si>
   <si>
     <t>Profile &gt; Notifications.</t>
@@ -1911,7 +1925,7 @@
     <t>A message confirms each change. The required notices stay on.</t>
   </si>
   <si>
-    <t>TC-114</t>
+    <t>TC-115</t>
   </si>
   <si>
     <t>Profile &gt; Appearance.</t>
@@ -1923,7 +1937,7 @@
     <t>The whole app changes at once and the choice is kept after signing in again.</t>
   </si>
   <si>
-    <t>TC-115</t>
+    <t>TC-116</t>
   </si>
   <si>
     <t>Profile &gt; Activity.</t>
@@ -1935,7 +1949,7 @@
     <t>It lists your own recent actions only.</t>
   </si>
   <si>
-    <t>TC-116</t>
+    <t>TC-117</t>
   </si>
   <si>
     <t>Signed in as each role.</t>
@@ -1947,7 +1961,7 @@
     <t>The basics and "Your account" always show. Med Ref, Checker, Approver, Accounting and Super Admin each see only their own guide; the link bar matches.</t>
   </si>
   <si>
-    <t>TC-117</t>
+    <t>TC-118</t>
   </si>
   <si>
     <t>Keeping records</t>
@@ -1964,7 +1978,7 @@
     <t>It lists by month the paid and disapproved receipts older than the period (not approved-but-unpaid ones), with their total and files. The CSV matches. Nothing is deleted or hidden.</t>
   </si>
   <si>
-    <t>TC-118</t>
+    <t>TC-119</t>
   </si>
   <si>
     <t>Keeping period set.</t>
@@ -1976,7 +1990,7 @@
     <t>It is refused. Only administrators can see it. Each preview and download is in the audit log.</t>
   </si>
   <si>
-    <t>TC-119</t>
+    <t>TC-120</t>
   </si>
   <si>
     <t>Phone</t>
@@ -1991,7 +2005,7 @@
     <t>Every screen fits the width with no sideways scrolling; buttons are easy to tap; the bottom menu stays in place.</t>
   </si>
   <si>
-    <t>TC-120</t>
+    <t>TC-121</t>
   </si>
   <si>
     <t>Display</t>
@@ -2006,7 +2020,7 @@
     <t>Text is easy to read everywhere; nothing is hidden (white on white or black on black).</t>
   </si>
   <si>
-    <t>TC-121</t>
+    <t>TC-122</t>
   </si>
   <si>
     <t>1. Scroll any screen.</t>
@@ -2015,7 +2029,7 @@
     <t>The browser window itself never scrolls: the top bar and side menu stay put.</t>
   </si>
   <si>
-    <t>TC-122</t>
+    <t>TC-123</t>
   </si>
   <si>
     <t>A receipt with evidence.</t>
@@ -2027,7 +2041,7 @@
     <t>Both are refused. Evidence is served only through the app to people allowed to see it.</t>
   </si>
   <si>
-    <t>TC-123</t>
+    <t>TC-124</t>
   </si>
   <si>
     <t>1. Check the address uses https and look at the cookie.</t>
@@ -2036,7 +2050,7 @@
     <t>Only one cookie is used; it is HttpOnly and Secure. No outside scripts or fonts load.</t>
   </si>
   <si>
-    <t>TC-124</t>
+    <t>TC-125</t>
   </si>
   <si>
     <t>A form with text boxes.</t>
@@ -2048,7 +2062,7 @@
     <t>It shows as plain text and does not run.</t>
   </si>
   <si>
-    <t>TC-125</t>
+    <t>TC-126</t>
   </si>
   <si>
     <t>A signed-in session.</t>
@@ -2060,7 +2074,7 @@
     <t>The change is refused (cross-site requests are rejected).</t>
   </si>
   <si>
-    <t>TC-126</t>
+    <t>TC-127</t>
   </si>
   <si>
     <t>1. Run node scripts/preflight.mjs.</t>
@@ -2069,7 +2083,7 @@
     <t>No BLOCKER is listed: production mode, https address, a mail account, a real Super Admin, no demo accounts, and a recent backup.</t>
   </si>
   <si>
-    <t>TC-127</t>
+    <t>TC-128</t>
   </si>
   <si>
     <t>1. Run the backup. Then restore it into a spare database with node scripts/restore.mjs ... --db reimsys_restore_test.</t>
@@ -2078,7 +2092,7 @@
     <t>The backup holds the database and the files. The restored copy has the same number of receipts.</t>
   </si>
   <si>
-    <t>TC-128</t>
+    <t>TC-129</t>
   </si>
   <si>
     <t>1. Run node scripts/healthcheck.mjs while the API is running, then stop the API and run it again.</t>
@@ -2087,7 +2101,7 @@
     <t>It prints nothing when healthy, and names the problem (API not answering, low disk, old backup, stuck emails) when not.</t>
   </si>
   <si>
-    <t>TC-129</t>
+    <t>TC-130</t>
   </si>
   <si>
     <t>The server cannot send email.</t>
@@ -3333,7 +3347,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4838,10 +4852,10 @@
         <v>44</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>175</v>
+        <v>197</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>301</v>
@@ -4911,7 +4925,7 @@
         <v>308</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>249</v>
+        <v>292</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>42</v>
@@ -4920,7 +4934,7 @@
         <v>44</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F39" s="13" t="s">
         <v>175</v>
@@ -4952,7 +4966,7 @@
         <v>312</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>43</v>
+        <v>249</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>42</v>
@@ -4961,10 +4975,10 @@
         <v>44</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F40" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>313</v>
@@ -5002,19 +5016,19 @@
         <v>44</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>317</v>
+        <v>157</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G41" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="H41" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="H41" s="8" t="s">
+      <c r="I41" s="8" t="s">
         <v>319</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>320</v>
       </c>
       <c r="J41" s="11" t="s">
         <v>162</v>
@@ -5031,7 +5045,7 @@
     </row>
     <row r="42" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>43</v>
@@ -5043,7 +5057,7 @@
         <v>44</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>165</v>
+        <v>321</v>
       </c>
       <c r="F42" s="10" t="s">
         <v>158</v>
@@ -5084,10 +5098,10 @@
         <v>44</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>175</v>
+        <v>165</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>326</v>
@@ -5116,10 +5130,10 @@
         <v>329</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>330</v>
+        <v>43</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>44</v>
@@ -5131,13 +5145,13 @@
         <v>175</v>
       </c>
       <c r="G44" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="H44" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="H44" s="8" t="s">
+      <c r="I44" s="8" t="s">
         <v>332</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>333</v>
       </c>
       <c r="J44" s="11" t="s">
         <v>162</v>
@@ -5154,10 +5168,10 @@
     </row>
     <row r="45" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="B45" s="8" t="s">
         <v>334</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>56</v>
@@ -5166,10 +5180,10 @@
         <v>44</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>335</v>
@@ -5198,28 +5212,28 @@
         <v>338</v>
       </c>
       <c r="B46" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="G46" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="C46" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F46" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G46" s="8" t="s">
+      <c r="H46" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="H46" s="8" t="s">
+      <c r="I46" s="8" t="s">
         <v>341</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>342</v>
       </c>
       <c r="J46" s="11" t="s">
         <v>162</v>
@@ -5236,13 +5250,13 @@
     </row>
     <row r="47" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="B47" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="B47" s="8" t="s">
-        <v>344</v>
-      </c>
       <c r="C47" s="8" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>64</v>
@@ -5250,17 +5264,17 @@
       <c r="E47" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>158</v>
+      <c r="F47" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G47" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="H47" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="H47" s="8" t="s">
+      <c r="I47" s="8" t="s">
         <v>346</v>
-      </c>
-      <c r="I47" s="8" t="s">
-        <v>347</v>
       </c>
       <c r="J47" s="11" t="s">
         <v>162</v>
@@ -5277,10 +5291,10 @@
     </row>
     <row r="48" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="B48" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>344</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>62</v>
@@ -5321,16 +5335,16 @@
         <v>352</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>62</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>317</v>
+        <v>157</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>158</v>
@@ -5362,7 +5376,7 @@
         <v>356</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>62</v>
@@ -5371,19 +5385,19 @@
         <v>44</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F50" s="13" t="s">
-        <v>175</v>
+        <v>321</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>309</v>
+        <v>357</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I50" s="8" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="J50" s="11" t="s">
         <v>162</v>
@@ -5400,25 +5414,25 @@
     </row>
     <row r="51" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>62</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E51" s="8" t="s">
         <v>197</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>360</v>
+        <v>313</v>
       </c>
       <c r="H51" s="8" t="s">
         <v>361</v>
@@ -5444,7 +5458,7 @@
         <v>363</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>364</v>
+        <v>348</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>62</v>
@@ -5453,19 +5467,19 @@
         <v>64</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G52" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="H52" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="H52" s="8" t="s">
+      <c r="I52" s="8" t="s">
         <v>366</v>
-      </c>
-      <c r="I52" s="8" t="s">
-        <v>367</v>
       </c>
       <c r="J52" s="11" t="s">
         <v>162</v>
@@ -5482,10 +5496,10 @@
     </row>
     <row r="53" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B53" s="8" t="s">
         <v>368</v>
-      </c>
-      <c r="B53" s="8" t="s">
-        <v>364</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>62</v>
@@ -5526,7 +5540,7 @@
         <v>372</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>62</v>
@@ -5535,10 +5549,10 @@
         <v>64</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="F54" s="13" t="s">
-        <v>175</v>
+        <v>157</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>373</v>
@@ -5567,19 +5581,19 @@
         <v>376</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F55" s="10" t="s">
-        <v>158</v>
+        <v>216</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>377</v>
@@ -5608,16 +5622,16 @@
         <v>380</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>317</v>
+        <v>157</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>158</v>
@@ -5649,7 +5663,7 @@
         <v>384</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>62</v>
@@ -5658,10 +5672,10 @@
         <v>64</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F57" s="13" t="s">
-        <v>175</v>
+        <v>321</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>385</v>
@@ -5690,10 +5704,10 @@
         <v>388</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>64</v>
@@ -5731,10 +5745,10 @@
         <v>392</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>64</v>
@@ -5772,28 +5786,28 @@
         <v>396</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>397</v>
+        <v>368</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E60" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F60" s="10" t="s">
-        <v>158</v>
+      <c r="F60" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G60" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="H60" s="8" t="s">
         <v>398</v>
       </c>
-      <c r="H60" s="8" t="s">
+      <c r="I60" s="8" t="s">
         <v>399</v>
-      </c>
-      <c r="I60" s="8" t="s">
-        <v>400</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>162</v>
@@ -5810,10 +5824,10 @@
     </row>
     <row r="61" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
+        <v>400</v>
+      </c>
+      <c r="B61" s="8" t="s">
         <v>401</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>397</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>76</v>
@@ -5828,13 +5842,13 @@
         <v>158</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="H61" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J61" s="11" t="s">
         <v>162</v>
@@ -5851,10 +5865,10 @@
     </row>
     <row r="62" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>76</v>
@@ -5863,13 +5877,13 @@
         <v>77</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F62" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="H62" s="8" t="s">
         <v>406</v>
@@ -5895,7 +5909,7 @@
         <v>408</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>76</v>
@@ -5904,19 +5918,19 @@
         <v>77</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F63" s="13" t="s">
-        <v>175</v>
+        <v>216</v>
+      </c>
+      <c r="F63" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>398</v>
+        <v>409</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>162</v>
@@ -5933,10 +5947,10 @@
     </row>
     <row r="64" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>76</v>
@@ -5951,13 +5965,13 @@
         <v>175</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="H64" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J64" s="11" t="s">
         <v>162</v>
@@ -5974,10 +5988,10 @@
     </row>
     <row r="65" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>76</v>
@@ -5992,7 +6006,7 @@
         <v>175</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>415</v>
+        <v>402</v>
       </c>
       <c r="H65" s="8" t="s">
         <v>416</v>
@@ -6018,7 +6032,7 @@
         <v>418</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>76</v>
@@ -6059,7 +6073,7 @@
         <v>422</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>76</v>
@@ -6068,10 +6082,10 @@
         <v>77</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="F67" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G67" s="8" t="s">
         <v>423</v>
@@ -6100,28 +6114,28 @@
         <v>426</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>76</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>250</v>
+        <v>427</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J68" s="11" t="s">
         <v>162</v>
@@ -6138,25 +6152,25 @@
     </row>
     <row r="69" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>84</v>
+        <v>401</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>157</v>
+        <v>321</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>430</v>
+        <v>250</v>
       </c>
       <c r="H69" s="8" t="s">
         <v>431</v>
@@ -6232,7 +6246,7 @@
         <v>85</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>158</v>
@@ -6273,10 +6287,10 @@
         <v>85</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F72" s="13" t="s">
-        <v>175</v>
+        <v>216</v>
+      </c>
+      <c r="F72" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G72" s="8" t="s">
         <v>442</v>
@@ -6355,10 +6369,10 @@
         <v>85</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="F74" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>450</v>
@@ -6393,10 +6407,10 @@
         <v>83</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>158</v>
@@ -6431,16 +6445,16 @@
         <v>84</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F76" s="13" t="s">
-        <v>190</v>
+        <v>321</v>
+      </c>
+      <c r="F76" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G76" s="8" t="s">
         <v>458</v>
@@ -6469,19 +6483,19 @@
         <v>461</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F77" s="10" t="s">
-        <v>158</v>
+      <c r="F77" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G77" s="8" t="s">
         <v>462</v>
@@ -6521,8 +6535,8 @@
       <c r="E78" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F78" s="13" t="s">
-        <v>175</v>
+      <c r="F78" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G78" s="8" t="s">
         <v>466</v>
@@ -6560,7 +6574,7 @@
         <v>64</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F79" s="13" t="s">
         <v>175</v>
@@ -6601,7 +6615,7 @@
         <v>64</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="F80" s="13" t="s">
         <v>175</v>
@@ -6639,13 +6653,13 @@
         <v>91</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="F81" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F81" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G81" s="8" t="s">
         <v>478</v>
@@ -6680,13 +6694,13 @@
         <v>91</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F82" s="13" t="s">
-        <v>190</v>
+        <v>321</v>
+      </c>
+      <c r="F82" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G82" s="8" t="s">
         <v>482</v>
@@ -6715,28 +6729,28 @@
         <v>485</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>486</v>
+        <v>92</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F83" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F83" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G83" s="8" t="s">
+        <v>486</v>
+      </c>
+      <c r="H83" s="8" t="s">
         <v>487</v>
       </c>
-      <c r="H83" s="8" t="s">
+      <c r="I83" s="8" t="s">
         <v>488</v>
-      </c>
-      <c r="I83" s="8" t="s">
-        <v>489</v>
       </c>
       <c r="J83" s="11" t="s">
         <v>162</v>
@@ -6753,10 +6767,10 @@
     </row>
     <row r="84" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
+        <v>489</v>
+      </c>
+      <c r="B84" s="8" t="s">
         <v>490</v>
-      </c>
-      <c r="B84" s="8" t="s">
-        <v>486</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>125</v>
@@ -6767,8 +6781,8 @@
       <c r="E84" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F84" s="13" t="s">
-        <v>175</v>
+      <c r="F84" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G84" s="8" t="s">
         <v>491</v>
@@ -6797,19 +6811,19 @@
         <v>494</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>156</v>
+        <v>64</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F85" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G85" s="8" t="s">
         <v>495</v>
@@ -6838,19 +6852,19 @@
         <v>498</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>126</v>
+        <v>490</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>44</v>
+        <v>156</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F86" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F86" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G86" s="8" t="s">
         <v>499</v>
@@ -6879,13 +6893,13 @@
         <v>502</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>503</v>
+        <v>126</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>125</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E87" s="8" t="s">
         <v>157</v>
@@ -6894,13 +6908,13 @@
         <v>158</v>
       </c>
       <c r="G87" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="H87" s="8" t="s">
         <v>504</v>
       </c>
-      <c r="H87" s="8" t="s">
+      <c r="I87" s="8" t="s">
         <v>505</v>
-      </c>
-      <c r="I87" s="8" t="s">
-        <v>506</v>
       </c>
       <c r="J87" s="11" t="s">
         <v>162</v>
@@ -6917,10 +6931,10 @@
     </row>
     <row r="88" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="B88" s="8" t="s">
         <v>507</v>
-      </c>
-      <c r="B88" s="8" t="s">
-        <v>503</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>125</v>
@@ -6929,10 +6943,10 @@
         <v>101</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F88" s="13" t="s">
-        <v>175</v>
+        <v>157</v>
+      </c>
+      <c r="F88" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G88" s="8" t="s">
         <v>508</v>
@@ -6961,19 +6975,19 @@
         <v>511</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="D89" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F89" s="10" t="s">
-        <v>158</v>
+        <v>165</v>
+      </c>
+      <c r="F89" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G89" s="8" t="s">
         <v>512</v>
@@ -7002,7 +7016,7 @@
         <v>515</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>107</v>
@@ -7017,13 +7031,13 @@
         <v>158</v>
       </c>
       <c r="G90" s="8" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="H90" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="I90" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>162</v>
@@ -7040,13 +7054,13 @@
     </row>
     <row r="91" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="D91" s="8" t="s">
         <v>101</v>
@@ -7054,11 +7068,11 @@
       <c r="E91" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F91" s="13" t="s">
-        <v>175</v>
+      <c r="F91" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="H91" s="8" t="s">
         <v>520</v>
@@ -7084,10 +7098,10 @@
         <v>522</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>101</v>
@@ -7096,7 +7110,7 @@
         <v>157</v>
       </c>
       <c r="F92" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G92" s="8" t="s">
         <v>523</v>
@@ -7125,10 +7139,10 @@
         <v>526</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>101</v>
@@ -7166,10 +7180,10 @@
         <v>530</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>29</v>
+        <v>507</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D94" s="8" t="s">
         <v>101</v>
@@ -7177,17 +7191,17 @@
       <c r="E94" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F94" s="10" t="s">
-        <v>158</v>
+      <c r="F94" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>237</v>
+        <v>531</v>
       </c>
       <c r="H94" s="8" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="I94" s="8" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>162</v>
@@ -7204,7 +7218,7 @@
     </row>
     <row r="95" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B95" s="8" t="s">
         <v>29</v>
@@ -7222,7 +7236,7 @@
         <v>158</v>
       </c>
       <c r="G95" s="8" t="s">
-        <v>534</v>
+        <v>237</v>
       </c>
       <c r="H95" s="8" t="s">
         <v>535</v>
@@ -7259,8 +7273,8 @@
       <c r="E96" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F96" s="13" t="s">
-        <v>175</v>
+      <c r="F96" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G96" s="8" t="s">
         <v>538</v>
@@ -7298,10 +7312,10 @@
         <v>101</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F97" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F97" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G97" s="8" t="s">
         <v>542</v>
@@ -7339,7 +7353,7 @@
         <v>101</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F98" s="10" t="s">
         <v>158</v>
@@ -7382,8 +7396,8 @@
       <c r="E99" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F99" s="13" t="s">
-        <v>190</v>
+      <c r="F99" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G99" s="8" t="s">
         <v>550</v>
@@ -7415,7 +7429,7 @@
         <v>29</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>101</v>
@@ -7424,16 +7438,16 @@
         <v>157</v>
       </c>
       <c r="F100" s="13" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>458</v>
+        <v>554</v>
       </c>
       <c r="H100" s="8" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="I100" s="8" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>162</v>
@@ -7450,7 +7464,7 @@
     </row>
     <row r="101" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>29</v>
@@ -7462,19 +7476,19 @@
         <v>101</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="F101" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="H101" s="8" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="I101" s="8" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="J101" s="11" t="s">
         <v>162</v>
@@ -7491,7 +7505,7 @@
     </row>
     <row r="102" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="8" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B102" s="8" t="s">
         <v>29</v>
@@ -7503,13 +7517,13 @@
         <v>101</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="F102" s="13" t="s">
         <v>190</v>
       </c>
       <c r="G102" s="8" t="s">
-        <v>560</v>
+        <v>462</v>
       </c>
       <c r="H102" s="8" t="s">
         <v>561</v>
@@ -7538,25 +7552,25 @@
         <v>29</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="F103" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F103" s="13" t="s">
+        <v>190</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>250</v>
+        <v>564</v>
       </c>
       <c r="H103" s="8" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="I103" s="8" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="J103" s="11" t="s">
         <v>162</v>
@@ -7573,25 +7587,25 @@
     </row>
     <row r="104" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D104" s="8" t="s">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="F104" s="13" t="s">
-        <v>175</v>
+        <v>321</v>
+      </c>
+      <c r="F104" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G104" s="8" t="s">
-        <v>567</v>
+        <v>250</v>
       </c>
       <c r="H104" s="8" t="s">
         <v>568</v>
@@ -7626,10 +7640,10 @@
         <v>101</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="F105" s="10" t="s">
-        <v>158</v>
+        <v>216</v>
+      </c>
+      <c r="F105" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G105" s="8" t="s">
         <v>571</v>
@@ -7658,28 +7672,28 @@
         <v>574</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>575</v>
+        <v>29</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F106" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G106" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="H106" s="8" t="s">
         <v>576</v>
       </c>
-      <c r="H106" s="8" t="s">
+      <c r="I106" s="8" t="s">
         <v>577</v>
-      </c>
-      <c r="I106" s="8" t="s">
-        <v>578</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>162</v>
@@ -7696,10 +7710,10 @@
     </row>
     <row r="107" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="B107" s="8" t="s">
         <v>579</v>
-      </c>
-      <c r="B107" s="8" t="s">
-        <v>575</v>
       </c>
       <c r="C107" s="8" t="s">
         <v>112</v>
@@ -7710,8 +7724,8 @@
       <c r="E107" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F107" s="13" t="s">
-        <v>175</v>
+      <c r="F107" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G107" s="8" t="s">
         <v>580</v>
@@ -7740,7 +7754,7 @@
         <v>583</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>112</v>
@@ -7749,10 +7763,10 @@
         <v>101</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F108" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="F108" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G108" s="8" t="s">
         <v>584</v>
@@ -7781,16 +7795,16 @@
         <v>587</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C109" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>158</v>
@@ -7822,28 +7836,28 @@
         <v>591</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>119</v>
+        <v>579</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E110" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F110" s="13" t="s">
-        <v>175</v>
+      <c r="F110" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>121</v>
+        <v>592</v>
       </c>
       <c r="H110" s="8" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="I110" s="8" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>162</v>
@@ -7860,7 +7874,7 @@
     </row>
     <row r="111" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B111" s="8" t="s">
         <v>119</v>
@@ -7874,11 +7888,11 @@
       <c r="E111" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F111" s="10" t="s">
-        <v>158</v>
+      <c r="F111" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>595</v>
+        <v>121</v>
       </c>
       <c r="H111" s="8" t="s">
         <v>596</v>
@@ -7915,8 +7929,8 @@
       <c r="E112" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F112" s="13" t="s">
-        <v>175</v>
+      <c r="F112" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G112" s="8" t="s">
         <v>599</v>
@@ -7951,7 +7965,7 @@
         <v>118</v>
       </c>
       <c r="D113" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E113" s="8" t="s">
         <v>157</v>
@@ -7960,13 +7974,13 @@
         <v>175</v>
       </c>
       <c r="G113" s="8" t="s">
-        <v>220</v>
+        <v>603</v>
       </c>
       <c r="H113" s="8" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="I113" s="8" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="J113" s="11" t="s">
         <v>162</v>
@@ -7983,7 +7997,7 @@
     </row>
     <row r="114" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="8" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B114" s="8" t="s">
         <v>119</v>
@@ -7998,10 +8012,10 @@
         <v>157</v>
       </c>
       <c r="F114" s="13" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G114" s="8" t="s">
-        <v>606</v>
+        <v>220</v>
       </c>
       <c r="H114" s="8" t="s">
         <v>607</v>
@@ -8036,7 +8050,7 @@
         <v>156</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="F115" s="13" t="s">
         <v>190</v>
@@ -8077,7 +8091,7 @@
         <v>156</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
       <c r="F116" s="13" t="s">
         <v>190</v>
@@ -8109,10 +8123,10 @@
         <v>617</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="D117" s="8" t="s">
         <v>156</v>
@@ -8150,28 +8164,28 @@
         <v>621</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>622</v>
+        <v>133</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D118" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E118" s="8" t="s">
         <v>157</v>
       </c>
       <c r="F118" s="13" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="G118" s="8" t="s">
+        <v>622</v>
+      </c>
+      <c r="H118" s="8" t="s">
         <v>623</v>
       </c>
-      <c r="H118" s="8" t="s">
+      <c r="I118" s="8" t="s">
         <v>624</v>
-      </c>
-      <c r="I118" s="8" t="s">
-        <v>625</v>
       </c>
       <c r="J118" s="11" t="s">
         <v>162</v>
@@ -8188,10 +8202,10 @@
     </row>
     <row r="119" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="B119" s="8" t="s">
         <v>626</v>
-      </c>
-      <c r="B119" s="8" t="s">
-        <v>622</v>
       </c>
       <c r="C119" s="8" t="s">
         <v>107</v>
@@ -8200,7 +8214,7 @@
         <v>101</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>317</v>
+        <v>157</v>
       </c>
       <c r="F119" s="13" t="s">
         <v>175</v>
@@ -8232,28 +8246,28 @@
         <v>630</v>
       </c>
       <c r="B120" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D120" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="F120" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="G120" s="8" t="s">
         <v>631</v>
       </c>
-      <c r="C120" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D120" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E120" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="F120" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="G120" s="8" t="s">
+      <c r="H120" s="8" t="s">
         <v>632</v>
       </c>
-      <c r="H120" s="8" t="s">
+      <c r="I120" s="8" t="s">
         <v>633</v>
-      </c>
-      <c r="I120" s="8" t="s">
-        <v>634</v>
       </c>
       <c r="J120" s="11" t="s">
         <v>162</v>
@@ -8270,31 +8284,31 @@
     </row>
     <row r="121" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
+        <v>634</v>
+      </c>
+      <c r="B121" s="8" t="s">
         <v>635</v>
       </c>
-      <c r="B121" s="8" t="s">
-        <v>636</v>
-      </c>
       <c r="C121" s="8" t="s">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="D121" s="8" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="E121" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="F121" s="13" t="s">
-        <v>175</v>
+      <c r="F121" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G121" s="8" t="s">
+        <v>636</v>
+      </c>
+      <c r="H121" s="8" t="s">
         <v>637</v>
       </c>
-      <c r="H121" s="8" t="s">
+      <c r="I121" s="8" t="s">
         <v>638</v>
-      </c>
-      <c r="I121" s="8" t="s">
-        <v>639</v>
       </c>
       <c r="J121" s="11" t="s">
         <v>162</v>
@@ -8311,10 +8325,10 @@
     </row>
     <row r="122" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
+        <v>639</v>
+      </c>
+      <c r="B122" s="8" t="s">
         <v>640</v>
-      </c>
-      <c r="B122" s="8" t="s">
-        <v>636</v>
       </c>
       <c r="C122" s="8" t="s">
         <v>118</v>
@@ -8329,13 +8343,13 @@
         <v>175</v>
       </c>
       <c r="G122" s="8" t="s">
-        <v>495</v>
+        <v>641</v>
       </c>
       <c r="H122" s="8" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="I122" s="8" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="J122" s="11" t="s">
         <v>162</v>
@@ -8352,25 +8366,25 @@
     </row>
     <row r="123" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>170</v>
+        <v>640</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>28</v>
+        <v>118</v>
       </c>
       <c r="D123" s="8" t="s">
         <v>156</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F123" s="10" t="s">
-        <v>158</v>
+        <v>197</v>
+      </c>
+      <c r="F123" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>644</v>
+        <v>499</v>
       </c>
       <c r="H123" s="8" t="s">
         <v>645</v>
@@ -8411,13 +8425,13 @@
         <v>158</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>121</v>
+        <v>648</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="I124" s="8" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="J124" s="11" t="s">
         <v>162</v>
@@ -8434,7 +8448,7 @@
     </row>
     <row r="125" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B125" s="8" t="s">
         <v>170</v>
@@ -8448,11 +8462,11 @@
       <c r="E125" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F125" s="13" t="s">
-        <v>175</v>
+      <c r="F125" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G125" s="8" t="s">
-        <v>651</v>
+        <v>121</v>
       </c>
       <c r="H125" s="8" t="s">
         <v>652</v>
@@ -8519,28 +8533,28 @@
         <v>658</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>137</v>
+        <v>28</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F127" s="10" t="s">
-        <v>158</v>
+        <v>170</v>
+      </c>
+      <c r="F127" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G127" s="8" t="s">
-        <v>141</v>
+        <v>659</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="I127" s="8" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="J127" s="11" t="s">
         <v>162</v>
@@ -8557,7 +8571,7 @@
     </row>
     <row r="128" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B128" s="8" t="s">
         <v>138</v>
@@ -8578,10 +8592,10 @@
         <v>141</v>
       </c>
       <c r="H128" s="8" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="I128" s="8" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="J128" s="11" t="s">
         <v>162</v>
@@ -8598,7 +8612,7 @@
     </row>
     <row r="129" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B129" s="8" t="s">
         <v>138</v>
@@ -8612,17 +8626,17 @@
       <c r="E129" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F129" s="13" t="s">
-        <v>175</v>
+      <c r="F129" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="G129" s="8" t="s">
         <v>141</v>
       </c>
       <c r="H129" s="8" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="I129" s="8" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="J129" s="11" t="s">
         <v>162</v>
@@ -8639,7 +8653,7 @@
     </row>
     <row r="130" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B130" s="8" t="s">
         <v>138</v>
@@ -8653,11 +8667,11 @@
       <c r="E130" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F130" s="10" t="s">
-        <v>158</v>
+      <c r="F130" s="13" t="s">
+        <v>175</v>
       </c>
       <c r="G130" s="8" t="s">
-        <v>668</v>
+        <v>141</v>
       </c>
       <c r="H130" s="8" t="s">
         <v>669</v>
@@ -8678,9 +8692,50 @@
         <v>1</v>
       </c>
     </row>
+    <row r="131" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="8" t="s">
+        <v>671</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="F131" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G131" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="H131" s="8" t="s">
+        <v>673</v>
+      </c>
+      <c r="I131" s="8" t="s">
+        <v>674</v>
+      </c>
+      <c r="J131" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="K131" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="L131" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="M131" s="11" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M130"/>
-  <conditionalFormatting sqref="J2:J130">
+  <autoFilter ref="A1:M131"/>
+  <conditionalFormatting sqref="J2:J131">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -8692,10 +8747,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="J10:J130">
+    <dataValidation type="list" sqref="J10:J131">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J130">
+    <dataValidation type="list" sqref="J2:J131">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8716,7 +8771,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>1</v>
@@ -8742,22 +8797,22 @@
         <v>21</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8765,23 +8820,23 @@
         <v>155</v>
       </c>
       <c r="B3" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A3)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A3)</f>
         <v>10</v>
       </c>
       <c r="C3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A3,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A3,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A3,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F3" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A3,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A3,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>10</v>
       </c>
       <c r="G3" s="16">
@@ -8794,23 +8849,23 @@
         <v>201</v>
       </c>
       <c r="B4" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A4)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A4)</f>
         <v>7</v>
       </c>
       <c r="C4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A4,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A4,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A4,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F4" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A4,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A4,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G4" s="16">
@@ -8823,23 +8878,23 @@
         <v>228</v>
       </c>
       <c r="B5" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A5)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A5)</f>
         <v>1</v>
       </c>
       <c r="C5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A5,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A5,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A5,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F5" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A5,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A5,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G5" s="16">
@@ -8852,23 +8907,23 @@
         <v>233</v>
       </c>
       <c r="B6" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A6)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A6)</f>
         <v>4</v>
       </c>
       <c r="C6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A6,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A6,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A6,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A6,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A6,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G6" s="16">
@@ -8881,23 +8936,23 @@
         <v>249</v>
       </c>
       <c r="B7" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A7)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A7)</f>
         <v>8</v>
       </c>
       <c r="C7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A7,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A7,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A7,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F7" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A7,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A7,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G7" s="16">
@@ -8910,23 +8965,23 @@
         <v>276</v>
       </c>
       <c r="B8" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A8)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A8,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A8,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A8,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F8" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A8,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A8,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G8" s="16">
@@ -8939,24 +8994,24 @@
         <v>292</v>
       </c>
       <c r="B9" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A9)</f>
-        <v>4</v>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A9)</f>
+        <v>5</v>
       </c>
       <c r="C9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A9,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A9,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A9,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A9,'Test cases'!$J$2:$J$130,"Not run")</f>
-        <v>4</v>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A9,'Test cases'!$J$2:$J$131,"Not run")</f>
+        <v>5</v>
       </c>
       <c r="G9" s="16">
         <f>IF(B9=0,0,C9/B9)</f>
@@ -8968,23 +9023,23 @@
         <v>43</v>
       </c>
       <c r="B10" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A10)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A10)</f>
         <v>4</v>
       </c>
       <c r="C10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A10,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A10,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A10,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A10,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A10,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G10" s="16">
@@ -8994,26 +9049,26 @@
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B11" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A11)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A11)</f>
         <v>2</v>
       </c>
       <c r="C11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A11,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A11,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A11,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F11" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A11,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A11,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G11" s="16">
@@ -9023,26 +9078,26 @@
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B12" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A12)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A12)</f>
         <v>1</v>
       </c>
       <c r="C12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A12,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A12,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A12,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A12,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A12,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G12" s="16">
@@ -9052,26 +9107,26 @@
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B13" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A13)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A13)</f>
         <v>5</v>
       </c>
       <c r="C13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A13,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A13,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A13,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A13,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A13,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>5</v>
       </c>
       <c r="G13" s="16">
@@ -9081,26 +9136,26 @@
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B14" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A14)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A14)</f>
         <v>8</v>
       </c>
       <c r="C14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A14,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A14,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A14,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A14,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A14,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G14" s="16">
@@ -9110,26 +9165,26 @@
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B15" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A15)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A15)</f>
         <v>9</v>
       </c>
       <c r="C15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A15,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A15,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A15,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A15,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A15,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>9</v>
       </c>
       <c r="G15" s="16">
@@ -9142,23 +9197,23 @@
         <v>84</v>
       </c>
       <c r="B16" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A16)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A16)</f>
         <v>8</v>
       </c>
       <c r="C16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A16,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A16,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A16,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A16,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A16,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G16" s="16">
@@ -9171,23 +9226,23 @@
         <v>92</v>
       </c>
       <c r="B17" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A17)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A17)</f>
         <v>6</v>
       </c>
       <c r="C17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A17,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A17,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A17,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A17,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A17,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>6</v>
       </c>
       <c r="G17" s="16">
@@ -9197,26 +9252,26 @@
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B18" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A18)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A18)</f>
         <v>3</v>
       </c>
       <c r="C18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A18,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A18,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A18,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A18,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A18,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G18" s="16">
@@ -9229,23 +9284,23 @@
         <v>126</v>
       </c>
       <c r="B19" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A19)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A19,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A19,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A19,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A19,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A19,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G19" s="16">
@@ -9255,26 +9310,26 @@
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="B20" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A20)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A20)</f>
         <v>7</v>
       </c>
       <c r="C20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A20,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A20,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A20,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A20,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A20,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G20" s="16">
@@ -9287,23 +9342,23 @@
         <v>29</v>
       </c>
       <c r="B21" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A21)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A21)</f>
         <v>12</v>
       </c>
       <c r="C21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A21,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A21,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A21,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A21,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A21,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>12</v>
       </c>
       <c r="G21" s="16">
@@ -9313,26 +9368,26 @@
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B22" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A22)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A22)</f>
         <v>4</v>
       </c>
       <c r="C22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A22,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A22,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A22,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A22,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A22,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G22" s="16">
@@ -9345,23 +9400,23 @@
         <v>119</v>
       </c>
       <c r="B23" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A23)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A23)</f>
         <v>7</v>
       </c>
       <c r="C23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A23,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A23,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A23,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A23,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A23,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G23" s="16">
@@ -9374,23 +9429,23 @@
         <v>133</v>
       </c>
       <c r="B24" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A24)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A24)</f>
         <v>1</v>
       </c>
       <c r="C24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A24,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A24,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A24,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A24,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A24,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G24" s="16">
@@ -9400,26 +9455,26 @@
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="B25" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A25)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A25)</f>
         <v>2</v>
       </c>
       <c r="C25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A25,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A25,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A25,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A25,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A25,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G25" s="16">
@@ -9429,26 +9484,26 @@
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="B26" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A26)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A26,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A26,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A26,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A26,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A26,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="16">
@@ -9458,26 +9513,26 @@
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="B27" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A27)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A27)</f>
         <v>2</v>
       </c>
       <c r="C27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A27,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A27,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A27,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A27,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A27,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G27" s="16">
@@ -9490,23 +9545,23 @@
         <v>170</v>
       </c>
       <c r="B28" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A28)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A28)</f>
         <v>4</v>
       </c>
       <c r="C28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A28,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A28,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A28,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F28" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A28,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A28,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G28" s="16">
@@ -9519,23 +9574,23 @@
         <v>138</v>
       </c>
       <c r="B29" s="15">
-        <f>COUNTIF('Test cases'!$B$2:$B$130,$A29)</f>
+        <f>COUNTIF('Test cases'!$B$2:$B$131,$A29)</f>
         <v>4</v>
       </c>
       <c r="C29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A29,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A29,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A29,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F29" s="15">
-        <f>COUNTIFS('Test cases'!$B$2:$B$130,$A29,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$B$2:$B$131,$A29,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G29" s="16">
@@ -9545,11 +9600,11 @@
     </row>
     <row r="30" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="B30" s="18">
         <f>SUM(B3:B29)</f>
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C30" s="18">
         <f>SUM(C3:C29)</f>
@@ -9565,7 +9620,7 @@
       </c>
       <c r="F30" s="18">
         <f>SUM(F3:F29)</f>
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G30" s="19">
         <f>IF(B30=0,0,C30/B30)</f>
@@ -9574,7 +9629,7 @@
     </row>
     <row r="32" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>1</v>
@@ -9600,22 +9655,22 @@
         <v>12</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>162</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="20" customFormat="1" x14ac:dyDescent="0.25">
@@ -9623,24 +9678,24 @@
         <v>158</v>
       </c>
       <c r="B34" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$130,A34)</f>
-        <v>64</v>
+        <f>COUNTIF('Test cases'!$F$2:$F$131,A34)</f>
+        <v>65</v>
       </c>
       <c r="C34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A34,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A34,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A34,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F34" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A34,'Test cases'!$J$2:$J$130,"Not run")</f>
-        <v>64</v>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A34,'Test cases'!$J$2:$J$131,"Not run")</f>
+        <v>65</v>
       </c>
       <c r="G34" s="22">
         <f>IF(B34=0,0,C34/B34)</f>
@@ -9652,23 +9707,23 @@
         <v>175</v>
       </c>
       <c r="B35" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$130,A35)</f>
+        <f>COUNTIF('Test cases'!$F$2:$F$131,A35)</f>
         <v>47</v>
       </c>
       <c r="C35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A35,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A35,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A35,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F35" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A35,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A35,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>47</v>
       </c>
       <c r="G35" s="22">
@@ -9681,23 +9736,23 @@
         <v>190</v>
       </c>
       <c r="B36" s="21">
-        <f>COUNTIF('Test cases'!$F$2:$F$130,A36)</f>
+        <f>COUNTIF('Test cases'!$F$2:$F$131,A36)</f>
         <v>18</v>
       </c>
       <c r="C36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Pass")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A36,'Test cases'!$J$2:$J$131,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Fail")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A36,'Test cases'!$J$2:$J$131,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Blocked")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A36,'Test cases'!$J$2:$J$131,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F36" s="21">
-        <f>COUNTIFS('Test cases'!$F$2:$F$130,$A36,'Test cases'!$J$2:$J$130,"Not run")</f>
+        <f>COUNTIFS('Test cases'!$F$2:$F$131,$A36,'Test cases'!$J$2:$J$131,"Not run")</f>
         <v>18</v>
       </c>
       <c r="G36" s="22">
@@ -9707,7 +9762,7 @@
     </row>
     <row r="38" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
     </row>
   </sheetData>
@@ -9730,19 +9785,19 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9750,16 +9805,16 @@
         <v>44</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9767,16 +9822,16 @@
         <v>64</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9784,16 +9839,16 @@
         <v>77</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9801,16 +9856,16 @@
         <v>85</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -9818,21 +9873,21 @@
         <v>101</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>